<commit_message>
docs: marcar 3.10–3.17 como Completo y actualizar el plan del epic
- Copia la versión del Excel del socio (septiembre 8, 33 stories: la
  ronda de feedback 3.10-3.17 sobre Epic A + el epic nuevo 4.1-4.9 de
  Dashboard/Mis deudas que se trabaja aparte, en otro worktree/sesión).
- Marca 3.10-3.17 como Completo (4.1-4.9 quedan Pendiente, no son de
  esta rama) y regenera roadmap.md con sync.py.
- Agrega la sección "Ronda de feedback del socio (3.10–3.17)" al plan
  del epic con el detalle y commit de cada story.
</commit_message>
<xml_diff>
--- a/docs/roadmap/Finance-BFF-Experience-Roadmap.xlsx
+++ b/docs/roadmap/Finance-BFF-Experience-Roadmap.xlsx
@@ -16,7 +16,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <color theme="1"/>
@@ -27,27 +27,8 @@
       <family val="2"/>
       <sz val="11"/>
     </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <family val="2"/>
-      <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -61,11 +42,21 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF3E8FF"/>
+        <fgColor theme="0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFEDE4F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDFF4F2"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -88,35 +79,77 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -414,24 +447,25 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M17"/>
+  <dimension ref="A1:M34"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="13.8"/>
   <cols>
-    <col width="24" customWidth="1" style="2" min="1" max="1"/>
-    <col width="8" customWidth="1" style="8" min="2" max="2"/>
-    <col width="28" customWidth="1" style="2" min="3" max="3"/>
-    <col width="55" customWidth="1" style="2" min="4" max="5"/>
-    <col width="60" customWidth="1" style="2" min="6" max="6"/>
-    <col width="55" customWidth="1" style="2" min="7" max="7"/>
-    <col width="40" customWidth="1" style="2" min="8" max="8"/>
-    <col width="28" customWidth="1" style="2" min="9" max="9"/>
-    <col width="35" customWidth="1" style="2" min="10" max="11"/>
-    <col width="10" customWidth="1" style="2" min="12" max="12"/>
-    <col width="12" customWidth="1" style="2" min="13" max="13"/>
-    <col width="8.88671875" customWidth="1" style="2" min="14" max="16384"/>
+    <col width="24" customWidth="1" style="5" min="1" max="1"/>
+    <col width="8" customWidth="1" style="4" min="2" max="2"/>
+    <col width="28" customWidth="1" style="5" min="3" max="3"/>
+    <col width="55" customWidth="1" style="5" min="4" max="5"/>
+    <col width="60" customWidth="1" style="5" min="6" max="6"/>
+    <col width="55" customWidth="1" style="5" min="7" max="7"/>
+    <col width="40" customWidth="1" style="5" min="8" max="8"/>
+    <col width="28" customWidth="1" style="5" min="9" max="9"/>
+    <col width="35" customWidth="1" style="5" min="10" max="11"/>
+    <col width="10" customWidth="1" style="5" min="12" max="12"/>
+    <col width="12" customWidth="1" style="5" min="13" max="13"/>
+    <col width="8.88671875" customWidth="1" style="5" min="14" max="14"/>
+    <col width="8.88671875" customWidth="1" style="5" min="15" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="1" s="1">
+    <row r="1" customFormat="1" s="4">
       <c r="A1" s="3" t="inlineStr">
         <is>
           <t>Epic</t>
@@ -498,477 +532,477 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="82.8" customHeight="1">
-      <c r="A2" s="4" t="inlineStr">
+    <row r="2" ht="53.1" customHeight="1">
+      <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="2" t="inlineStr">
         <is>
           <t>2.1</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="1" t="inlineStr">
         <is>
           <t>Rediseñar el Hero</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="1" t="inlineStr">
         <is>
           <t>El Hero comunica la propuesta de valor, pero la diferenciación frente a otras aplicaciones financieras no es inmediata. El producto tiene menos protagonismo del deseado y la jerarquía visual puede hacer que la usuaria invierta más tiempo del necesario para entender qué ofrece Finance BFF y por qué debería confiar en la plataforma.</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="E2" s="1" t="inlineStr">
         <is>
           <t>Desde los primeros segundos la usuaria debe comprender que Finance BFF es una guía financiera paso a paso. El Hero debe transmitir cercanía, confianza y claridad, mostrando el producto como protagonista y motivando a iniciar el registro sin necesidad de hacer scroll.</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="1" t="inlineStr">
         <is>
           <t>Como una mujer que visita Finance BFF por primera vez y siente que no tiene claridad sobre sus finanzas, quiero entender inmediatamente qué es Finance BFF, cómo me ayudará y por qué es diferente, para sentir confianza y querer empezar mi proceso de organización financiera.</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="G2" s="1" t="inlineStr">
         <is>
           <t>Rediseñar completamente el Hero incorporando navegación, headline, subtítulo, CTA principal, CTA secundario, mockup del producto y diseño responsive.</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
+      <c r="H2" s="1" t="inlineStr">
         <is>
           <t>Conservar la identidad visual y la paleta de rosados. El mockup debe ser protagonista y el CTA principal debe tener la mayor jerarquía visual.</t>
         </is>
       </c>
-      <c r="I2" s="4" t="inlineStr">
+      <c r="I2" s="1" t="inlineStr">
         <is>
           <t>Comunicar claramente la propuesta de valor e incrementar la conversión.</t>
         </is>
       </c>
-      <c r="J2" s="4" t="inlineStr">
+      <c r="J2" s="1" t="inlineStr">
         <is>
           <t>La usuaria comprende el valor del producto y quiere continuar.</t>
         </is>
       </c>
-      <c r="K2" s="4" t="inlineStr">
+      <c r="K2" s="1" t="inlineStr">
         <is>
           <t>La propuesta de valor se entiende en pocos segundos.</t>
         </is>
       </c>
-      <c r="L2" s="4" t="inlineStr">
+      <c r="L2" s="1" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="M2" s="4" t="inlineStr">
+      <c r="M2" s="1" t="inlineStr">
         <is>
           <t>Completo</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="69" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
+    <row r="3" ht="44.1" customHeight="1">
+      <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>2.2</t>
         </is>
       </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="C3" s="1" t="inlineStr">
         <is>
           <t>Mockup principal de Amy</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
+      <c r="D3" s="1" t="inlineStr">
         <is>
           <t>Actualmente el producto no tiene suficiente protagonismo dentro del Hero, lo que dificulta que la usuaria imagine cómo será la experiencia después del registro. La propuesta depende demasiado del texto y poco de la demostración visual.</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="E3" s="1" t="inlineStr">
         <is>
           <t>La usuaria debe visualizar inmediatamente una versión real del producto y entender que Amy interpreta la información financiera y la guía con recomendaciones personalizadas. El mockup debe generar confianza y reducir la incertidumbre sobre lo que recibirá.</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
+      <c r="F3" s="1" t="inlineStr">
         <is>
           <t>Como una mujer que está evaluando si Finance BFF realmente puede ayudarla, quiero ver el producto desde el primer momento para imaginar cómo sería utilizar la plataforma y entender que recibiré acompañamiento más allá de un simple registro de gastos.</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="1" t="inlineStr">
         <is>
           <t>Crear un mockup de alta fidelidad con información financiera realista, recomendaciones de Amy y componentes auténticos del producto.</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="1" t="inlineStr">
         <is>
           <t>El mockup debe sentirse premium, ser coherente con la marca y convertirse en el principal apoyo visual del Hero.</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="I3" s="1" t="inlineStr">
         <is>
           <t>Hacer tangible el producto antes del registro.</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="J3" s="1" t="inlineStr">
         <is>
           <t>La usuaria visualiza claramente la experiencia.</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="K3" s="1" t="inlineStr">
         <is>
           <t>El mockup comunica el funcionamiento del producto.</t>
         </is>
       </c>
-      <c r="L3" s="4" t="inlineStr">
+      <c r="L3" s="1" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="M3" s="1" t="inlineStr">
         <is>
           <t>Completo</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="55.2" customHeight="1">
-      <c r="A4" s="4" t="inlineStr">
+    <row r="4" ht="35.25" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>2.3</t>
         </is>
       </c>
-      <c r="C4" s="4" t="inlineStr">
+      <c r="C4" s="1" t="inlineStr">
         <is>
           <t>CTA principal</t>
         </is>
       </c>
-      <c r="D4" s="4" t="inlineStr">
+      <c r="D4" s="1" t="inlineStr">
         <is>
           <t>El siguiente paso no destaca con suficiente fuerza y la usuaria puede perder algunos segundos identificando cuál es la acción principal que debe realizar para comenzar.</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
+      <c r="E4" s="1" t="inlineStr">
         <is>
           <t>La acción principal debe ser evidente desde el primer vistazo. El CTA debe transmitir seguridad, eliminar dudas y motivar el registro sin competir con otros elementos visuales.</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="F4" s="1" t="inlineStr">
         <is>
           <t>Como una mujer que ya entendió el valor de Finance BFF, quiero identificar inmediatamente cuál es el siguiente paso para comenzar, sin sentir dudas o confusión, para iniciar mi proceso con seguridad y sin fricción.</t>
         </is>
       </c>
-      <c r="G4" s="4" t="inlineStr">
+      <c r="G4" s="1" t="inlineStr">
         <is>
           <t>Crear un CTA principal dominante y un CTA secundario para iniciar sesión, manteniendo consistencia en todos los dispositivos.</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
+      <c r="H4" s="1" t="inlineStr">
         <is>
           <t>Ubicar el CTA cerca de la propuesta de valor y mantener una jerarquía visual clara.</t>
         </is>
       </c>
-      <c r="I4" s="4" t="inlineStr">
+      <c r="I4" s="1" t="inlineStr">
         <is>
           <t>Incrementar la conversión.</t>
         </is>
       </c>
-      <c r="J4" s="4" t="inlineStr">
+      <c r="J4" s="1" t="inlineStr">
         <is>
           <t>La usuaria sabe exactamente qué hacer.</t>
         </is>
       </c>
-      <c r="K4" s="4" t="inlineStr">
+      <c r="K4" s="1" t="inlineStr">
         <is>
           <t>El CTA es el elemento de mayor protagonismo después del titular.</t>
         </is>
       </c>
-      <c r="L4" s="4" t="inlineStr">
+      <c r="L4" s="1" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
+      <c r="M4" s="1" t="inlineStr">
         <is>
           <t>Completo</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="69" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+    <row r="5" ht="44.1" customHeight="1">
+      <c r="A5" s="1" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>2.4</t>
         </is>
       </c>
-      <c r="C5" s="4" t="inlineStr">
+      <c r="C5" s="1" t="inlineStr">
         <is>
           <t>Header y navegación</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="1" t="inlineStr">
         <is>
           <t>La navegación actual puede evolucionar para orientar mejor a usuarias nuevas y recurrentes, manteniendo el foco en la conversión sin generar distracciones.</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="1" t="inlineStr">
         <is>
           <t>La navegación debe sentirse simple, intuitiva y organizada. Debe facilitar el acceso a la información esencial y al inicio de sesión sin quitar protagonismo al Hero.</t>
         </is>
       </c>
-      <c r="F5" s="4" t="inlineStr">
+      <c r="F5" s="1" t="inlineStr">
         <is>
           <t>Como una mujer que está explorando Finance BFF por primera vez, quiero encontrar una navegación clara y sencilla que me permita moverme por la página y acceder fácilmente al inicio de sesión si ya tengo una cuenta, para sentir que la plataforma está bien organizada.</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="1" t="inlineStr">
         <is>
           <t>Construir un header limpio con logo, enlaces esenciales y botón de iniciar sesión.</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="1" t="inlineStr">
         <is>
           <t>Mantener simplicidad y coherencia visual.</t>
         </is>
       </c>
-      <c r="I5" s="4" t="inlineStr">
+      <c r="I5" s="1" t="inlineStr">
         <is>
           <t>Facilitar la exploración.</t>
         </is>
       </c>
-      <c r="J5" s="4" t="inlineStr">
+      <c r="J5" s="1" t="inlineStr">
         <is>
           <t>La navegación transmite orden y confianza.</t>
         </is>
       </c>
-      <c r="K5" s="4" t="inlineStr">
+      <c r="K5" s="1" t="inlineStr">
         <is>
           <t>La usuaria encuentra rápidamente lo que necesita.</t>
         </is>
       </c>
-      <c r="L5" s="4" t="inlineStr">
+      <c r="L5" s="1" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="M5" s="4" t="inlineStr">
+      <c r="M5" s="1" t="inlineStr">
         <is>
           <t>Completo</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="69" customHeight="1">
-      <c r="A6" s="4" t="inlineStr">
+    <row r="6" ht="44.1" customHeight="1">
+      <c r="A6" s="1" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>2.5</t>
         </is>
       </c>
-      <c r="C6" s="4" t="inlineStr">
+      <c r="C6" s="1" t="inlineStr">
         <is>
           <t>Animaciones del Hero</t>
         </is>
       </c>
-      <c r="D6" s="4" t="inlineStr">
+      <c r="D6" s="1" t="inlineStr">
         <is>
           <t>La experiencia es principalmente estática, por lo que la calidad percibida puede ser inferior al valor real del producto.</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
+      <c r="E6" s="1" t="inlineStr">
         <is>
           <t>La interfaz debe sentirse viva mediante microanimaciones elegantes que acompañen la interacción sin distraer ni afectar el rendimiento.</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="F6" s="1" t="inlineStr">
         <is>
           <t>Como una mujer que está evaluando si puede confiar en Finance BFF, quiero que la página tenga movimientos y transiciones suaves que hagan la experiencia más agradable, para percibir el producto como moderno y profesional sin distraerme del contenido principal.</t>
         </is>
       </c>
-      <c r="G6" s="4" t="inlineStr">
+      <c r="G6" s="1" t="inlineStr">
         <is>
           <t>Incorporar microanimaciones al cargar el Hero y durante las interacciones clave.</t>
         </is>
       </c>
-      <c r="H6" s="4" t="inlineStr">
+      <c r="H6" s="1" t="inlineStr">
         <is>
           <t>Las animaciones deben reforzar la experiencia y nunca convertirse en el foco.</t>
         </is>
       </c>
-      <c r="I6" s="4" t="inlineStr">
+      <c r="I6" s="1" t="inlineStr">
         <is>
           <t>Incrementar la percepción de calidad.</t>
         </is>
       </c>
-      <c r="J6" s="4" t="inlineStr">
+      <c r="J6" s="1" t="inlineStr">
         <is>
           <t>La experiencia se siente moderna.</t>
         </is>
       </c>
-      <c r="K6" s="4" t="inlineStr">
+      <c r="K6" s="1" t="inlineStr">
         <is>
           <t>Las animaciones no afectan el rendimiento.</t>
         </is>
       </c>
-      <c r="L6" s="4" t="inlineStr">
+      <c r="L6" s="1" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="M6" s="4" t="inlineStr">
+      <c r="M6" s="1" t="inlineStr">
         <is>
           <t>Completo</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="55.2" customHeight="1">
-      <c r="A7" s="4" t="inlineStr">
+    <row r="7" ht="35.25" customHeight="1">
+      <c r="A7" s="1" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>2.6</t>
         </is>
       </c>
-      <c r="C7" s="4" t="inlineStr">
+      <c r="C7" s="1" t="inlineStr">
         <is>
           <t>Responsive del Hero</t>
         </is>
       </c>
-      <c r="D7" s="4" t="inlineStr">
+      <c r="D7" s="1" t="inlineStr">
         <is>
           <t>La experiencia puede mejorar para garantizar que el mensaje conserve la misma claridad y jerarquía en cualquier tamaño de pantalla.</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E7" s="1" t="inlineStr">
         <is>
           <t>Sin importar el dispositivo, la usuaria debe recibir exactamente la misma propuesta de valor y una experiencia visual consistente.</t>
         </is>
       </c>
-      <c r="F7" s="4" t="inlineStr">
+      <c r="F7" s="1" t="inlineStr">
         <is>
           <t>Como una mujer que puede descubrir Finance BFF desde su celular, tablet o computador, quiero recibir una experiencia consistente sin importar el dispositivo que esté utilizando, para comprender la propuesta de valor con la misma facilidad.</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="1" t="inlineStr">
         <is>
           <t>Optimizar completamente el Hero para desktop, tablet y móvil.</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="1" t="inlineStr">
         <is>
           <t>Conservar jerarquía, legibilidad y paleta de colores.</t>
         </is>
       </c>
-      <c r="I7" s="4" t="inlineStr">
+      <c r="I7" s="1" t="inlineStr">
         <is>
           <t>Garantizar consistencia.</t>
         </is>
       </c>
-      <c r="J7" s="4" t="inlineStr">
+      <c r="J7" s="1" t="inlineStr">
         <is>
           <t>La experiencia es igual de clara en cualquier dispositivo.</t>
         </is>
       </c>
-      <c r="K7" s="4" t="inlineStr">
+      <c r="K7" s="1" t="inlineStr">
         <is>
           <t>No existen problemas de visualización.</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="L7" s="1" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="M7" s="4" t="inlineStr">
+      <c r="M7" s="1" t="inlineStr">
         <is>
           <t>Completo</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="69" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
+    <row r="8" ht="44.1" customHeight="1">
+      <c r="A8" s="1" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
         </is>
       </c>
-      <c r="B8" s="6" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>2.7</t>
         </is>
       </c>
-      <c r="C8" s="4" t="inlineStr">
+      <c r="C8" s="1" t="inlineStr">
         <is>
           <t>Optimización emocional del Hero</t>
         </is>
       </c>
-      <c r="D8" s="4" t="inlineStr">
+      <c r="D8" s="1" t="inlineStr">
         <is>
           <t>El Hero comunica beneficios funcionales, pero aún existe una oportunidad para conectar emocionalmente con mujeres que sienten frustración o ansiedad por sus finanzas.</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
+      <c r="E8" s="1" t="inlineStr">
         <is>
           <t>La usuaria debe sentir que Finance BFF comprende su situación antes de hablarle de funcionalidades. La conexión emocional debe generar confianza y hacer que la plataforma se perciba cercana y humana.</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="F8" s="1" t="inlineStr">
         <is>
           <t>Como una mujer que durante mucho tiempo ha sentido frustración o desorden con sus finanzas, quiero sentir desde los primeros segundos que Finance BFF comprende mi situación y me habla de una manera cercana y empática, para confiar en que realmente puede acompañarme.</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="1" t="inlineStr">
         <is>
           <t>Refinar el contenido, imágenes y mensajes para reforzar empatía y acompañamiento.</t>
         </is>
       </c>
-      <c r="H8" s="4" t="inlineStr">
+      <c r="H8" s="1" t="inlineStr">
         <is>
           <t>La emoción debe anteceder a la explicación funcional.</t>
         </is>
       </c>
-      <c r="I8" s="4" t="inlineStr">
+      <c r="I8" s="1" t="inlineStr">
         <is>
           <t>Generar conexión emocional.</t>
         </is>
       </c>
-      <c r="J8" s="4" t="inlineStr">
+      <c r="J8" s="1" t="inlineStr">
         <is>
           <t>La usuaria siente que Finance BFF fue creado para ella.</t>
         </is>
       </c>
-      <c r="K8" s="4" t="inlineStr">
+      <c r="K8" s="1" t="inlineStr">
         <is>
           <t>El Hero transmite cercanía y confianza.</t>
         </is>
       </c>
-      <c r="L8" s="4" t="inlineStr">
+      <c r="L8" s="1" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="M8" s="4" t="inlineStr">
+      <c r="M8" s="1" t="inlineStr">
         <is>
           <t>Completo</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="120" customHeight="1">
-      <c r="A9" s="5" t="inlineStr">
+    <row r="9" ht="76.8" customFormat="1" customHeight="1" s="8">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
         </is>
@@ -978,64 +1012,64 @@
           <t>3.1</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Guardar progreso y permitir volver atrás</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Durante el onboarding la usuaria puede avanzar entre varias pantallas, pero la experiencia no deja suficientemente explícito que su progreso se conserva si necesita salir. Además, el botón para regresar no está presente de forma consistente en todos los pasos.</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>La usuaria debe poder completar el onboarding a su ritmo. Todo dato confirmado o ingresado debe guardarse automáticamente y cada paso debe permitir volver atrás sin perder información ni obligarla a comenzar de nuevo.</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>Como una mujer que está organizando sus finanzas por primera vez y puede no tener tiempo para completar todo el proceso en una sola sesión, quiero que Finance BFF guarde automáticamente lo que voy haciendo y me permita regresar a pasos anteriores, para avanzar a mi ritmo sin miedo a perder información. y que me avise que eso va a pasar.</t>
         </is>
       </c>
-      <c r="G9" s="5" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>Implementar guardado automático durante todo el onboarding. Al volver a ingresar, llevar a la usuaria al último paso pendiente con la información previamente diligenciada. Incluir una acción Atrás en todos los pasos donde exista una pantalla anterior y conservar los datos al navegar entre pasos.</t>
         </is>
       </c>
-      <c r="H9" s="5" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>El guardado debe sentirse automático y silencioso, sin interrumpir el flujo. Evitar mensajes técnicos. Si se muestra confirmación, usar microcopy breve como 'Guardado'. La acción Atrás debe ser secundaria frente al CTA principal.</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>Reducir abandono del onboarding y facilitar que más usuarias lo completen.</t>
         </is>
       </c>
-      <c r="J9" s="5" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>La usuaria puede interrumpir y retomar el proceso sin perder avances ni repetir información.</t>
         </is>
       </c>
-      <c r="K9" s="5" t="inlineStr">
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>Salir y regresar conserva los datos y el paso alcanzado. Todos los pasos aplicables permiten volver atrás sin pérdida de información.</t>
         </is>
       </c>
-      <c r="L9" s="5" t="inlineStr">
+      <c r="L9" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="M9" s="5" t="inlineStr">
+      <c r="M9" s="6" t="inlineStr">
         <is>
           <t>Completo</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="120" customHeight="1">
-      <c r="A10" s="5" t="inlineStr">
+    <row r="10" ht="76.8" customFormat="1" customHeight="1" s="8">
+      <c r="A10" s="6" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
         </is>
@@ -1045,64 +1079,64 @@
           <t>3.2</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
         <is>
           <t>Formato inteligente para valores de dinero</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="6" t="inlineStr">
         <is>
           <t>Los campos monetarios no mantienen una presentación consistente mientras la usuaria escribe y algunos inputs muestran controles nativos con flechas para aumentar o disminuir números.</t>
         </is>
       </c>
-      <c r="E10" s="5" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>Todos los valores de dinero deben ser fáciles de leer desde el momento en que se ingresan, mostrando el signo $ y separadores de miles de forma automática, sin controles numéricos que generen ruido visual.</t>
         </is>
       </c>
-      <c r="F10" s="5" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>Como una mujer que está ingresando varios valores de ingresos, gastos, cajitas y ahorros, quiero ver los montos en un formato claro mientras los escribo, para evitar errores y entender rápidamente las cantidades que estoy registrando.</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Aplicar formato monetario en todos los campos de dinero del producto: signo $ y puntos como separadores de miles. El formato debe actualizarse mientras se escribe. Eliminar las flechas nativas de incremento y decremento de los inputs numéricos y mantener el campo abierto para escritura directa.</t>
         </is>
       </c>
-      <c r="H10" s="5" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>El formato debe ayudar a leer, no dificultar la edición. Mantener consistencia en onboarding, dashboard y módulos posteriores.</t>
         </is>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>Reducir errores de digitación y mejorar la comprensión de la información financiera.</t>
         </is>
       </c>
-      <c r="J10" s="5" t="inlineStr">
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>La usuaria interpreta los montos de inmediato y encuentra una experiencia consistente en toda la plataforma.</t>
         </is>
       </c>
-      <c r="K10" s="5" t="inlineStr">
+      <c r="K10" s="6" t="inlineStr">
         <is>
           <t>Todos los campos monetarios aplicables muestran $ y separadores de miles y ninguno presenta controles nativos de incremento/decremento.</t>
         </is>
       </c>
-      <c r="L10" s="5" t="inlineStr">
+      <c r="L10" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="M10" s="5" t="inlineStr">
+      <c r="M10" s="6" t="inlineStr">
         <is>
           <t>Completo</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="120" customHeight="1">
-      <c r="A11" s="5" t="inlineStr">
+    <row r="11" ht="76.8" customFormat="1" customHeight="1" s="8">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
         </is>
@@ -1112,64 +1146,64 @@
           <t>3.3</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Amy Detective reconoce primero el progreso</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>En el Happy Path la usuaria no tiene deudas y cuenta con capacidad para ahorrar, pero Amy Detective abre con un mensaje de alerta sobre el porcentaje de gastos fijos. El tono puede hacer que un escenario positivo se perciba como un problema.</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Amy debe reconocer primero lo que la usuaria está haciendo bien y después mostrar oportunidades de mejora. En este escenario debe celebrar que no tiene deudas y que existe margen para organizar su ahorro antes de hablar de optimización de gastos.</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>Como una mujer que acaba de compartir toda su información financiera y descubre que no tiene deudas y sí tiene capacidad de ahorro, quiero que Amy reconozca ese avance antes de señalar oportunidades de mejora, para sentir motivación y no interpretar mi situación como algo negativo.</t>
         </is>
       </c>
-      <c r="G11" s="5" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
         <is>
           <t>Reescribir el estado de Amy Detective para el Happy Path. Abrir con una felicitación o reconocimiento positivo. Después explicar de manera tranquila que los gastos fijos representan una parte importante de los ingresos y que Amy puede ayudar a revisar si existe espacio para liberar aún más dinero. Mantener la opción de revisar gastos o continuar.</t>
         </is>
       </c>
-      <c r="H11" s="5" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>Evitar lenguaje de alarma como '¡Oops!' cuando no existe una situación crítica. Amy debe sentirse como una BFF que reconoce avances y luego acompaña a mejorar.</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>Fortalecer la relación emocional con Amy y evitar ansiedad innecesaria.</t>
         </is>
       </c>
-      <c r="J11" s="5" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>La usuaria entiende que está en una buena posición y percibe la revisión de gastos como una oportunidad, no como una advertencia.</t>
         </is>
       </c>
-      <c r="K11" s="5" t="inlineStr">
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>El mensaje comienza reconociendo el escenario positivo y la oportunidad de optimización aparece como segundo mensaje.</t>
         </is>
       </c>
-      <c r="L11" s="5" t="inlineStr">
+      <c r="L11" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="M11" s="5" t="inlineStr">
+      <c r="M11" s="6" t="inlineStr">
         <is>
           <t>Completo</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="120" customHeight="1">
-      <c r="A12" s="5" t="inlineStr">
+    <row r="12" ht="76.8" customFormat="1" customHeight="1" s="8">
+      <c r="A12" s="6" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
         </is>
@@ -1179,64 +1213,64 @@
           <t>3.4</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="6" t="inlineStr">
         <is>
           <t>Explicar claramente el punto de partida del ahorro</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="6" t="inlineStr">
         <is>
           <t>La pantalla 'Este es tu punto de partida' muestra cálculos y tres opciones de ahorro, pero no explica con suficiente claridad qué hizo Amy con la información registrada, de dónde sale el dinero disponible ni qué decisión debe tomar la usuaria.</t>
         </is>
       </c>
-      <c r="E12" s="5" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>Antes de pedir una elección, Amy debe resumir en lenguaje sencillo cuánto dinero queda realmente disponible después de compromisos, cómo llegó a ese resultado y por qué propone diferentes niveles de ahorro.</t>
         </is>
       </c>
-      <c r="F12" s="5" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>Como una mujer que acaba de registrar ingresos, gastos y cajitas, quiero entender cuánto dinero me queda disponible y por qué Amy me recomienda ciertos montos de ahorro, para elegir una opción con confianza y sin sentir que estoy escogiendo números al azar.</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr">
         <is>
           <t>Reorganizar la pantalla para explicar la secuencia del cálculo antes de mostrar las opciones. Mostrar claramente: dinero disponible después de gastos, reserva mensual para cajitas y monto realmente disponible para decidir. Después presentar las alternativas de ahorro explicando la diferencia entre recomendada, intermedia y flexible y cuánto dinero libre queda en cada caso.</t>
         </is>
       </c>
-      <c r="H12" s="5" t="inlineStr">
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>Priorizar comprensión sobre cantidad de información. Los números principales deben tener jerarquía visual y el lenguaje debe explicar decisiones, no fórmulas.</t>
         </is>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>Aumentar la confianza en las recomendaciones de Amy y facilitar la selección del plan de ahorro.</t>
         </is>
       </c>
-      <c r="J12" s="5" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>La usuaria entiende de dónde sale su capacidad de ahorro, qué está eligiendo y cómo afecta su dinero disponible.</t>
         </is>
       </c>
-      <c r="K12" s="5" t="inlineStr">
+      <c r="K12" s="6" t="inlineStr">
         <is>
           <t>Una usuaria puede explicar con sus propias palabras de dónde sale el monto disponible y la diferencia entre las tres opciones antes de continuar.</t>
         </is>
       </c>
-      <c r="L12" s="5" t="inlineStr">
+      <c r="L12" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="M12" s="5" t="inlineStr">
+      <c r="M12" s="6" t="inlineStr">
         <is>
           <t>Completo</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="120" customHeight="1">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="13" ht="76.8" customFormat="1" customHeight="1" s="8">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
         </is>
@@ -1246,64 +1280,64 @@
           <t>3.5</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Mostrar dinero restante al crear bolsitas</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>Durante la creación de bolsitas existe un indicador de dinero disponible para repartir, pero pierde protagonismo a medida que se agregan bolsitas. Cuando el monto llega a $0 se utiliza un estado naranja que puede interpretarse como advertencia.</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>La usuaria debe saber en todo momento cuánto dinero de su ahorro mensual ya distribuyó y cuánto le queda por asignar. Llegar a $0 debe sentirse como completar exitosamente la organización del ahorro.</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
         <is>
           <t>Como una mujer que está repartiendo por primera vez su ahorro entre diferentes propósitos, quiero ver claramente cuánto dinero me queda por distribuir después de cada bolsita, para organizarlo sin pasarme del límite y sentir satisfacción cuando termino.</t>
         </is>
       </c>
-      <c r="G13" s="5" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Mantener visible y con alta jerarquía el saldo restante durante toda la creación de bolsitas. Actualizarlo en tiempo real después de agregar, editar o eliminar una bolsita. Cuando llegue a $0, reemplazar el estado de advertencia por un estado positivo con un mensaje como '¡Listo! Repartiste todo tu ahorro mensual' y habilitar claramente la continuación.</t>
         </is>
       </c>
-      <c r="H13" s="5" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>No usar naranja, rojo ni lenguaje de error cuando el dinero fue distribuido correctamente. El estado final puede incluir una microcelebración coherente con la marca.</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr">
         <is>
           <t>Facilitar la distribución del ahorro y reforzar la sensación de progreso.</t>
         </is>
       </c>
-      <c r="J13" s="5" t="inlineStr">
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>La usuaria sabe cuánto le queda por repartir en cada momento y entiende que llegar a $0 significa que completó el paso.</t>
         </is>
       </c>
-      <c r="K13" s="5" t="inlineStr">
+      <c r="K13" s="6" t="inlineStr">
         <is>
           <t>El saldo restante se actualiza inmediatamente y el estado de $0 se presenta como éxito, no como alerta.</t>
         </is>
       </c>
-      <c r="L13" s="5" t="inlineStr">
+      <c r="L13" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="M13" s="5" t="inlineStr">
+      <c r="M13" s="6" t="inlineStr">
         <is>
           <t>Completo</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="120" customHeight="1">
-      <c r="A14" s="5" t="inlineStr">
+    <row r="14" ht="76.8" customFormat="1" customHeight="1" s="8">
+      <c r="A14" s="6" t="inlineStr">
         <is>
           <t>Acompañamiento después del onboarding</t>
         </is>
@@ -1313,64 +1347,64 @@
           <t>3.6</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C14" s="6" t="inlineStr">
         <is>
           <t>Convertir Mis finanzas en un plan de acción</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D14" s="6" t="inlineStr">
         <is>
           <t>Al terminar el onboarding la usuaria llega a un dashboard con información financiera completa, pero no recibe suficiente orientación sobre qué hacer con esos números ni cuál debería ser su siguiente acción.</t>
         </is>
       </c>
-      <c r="E14" s="5" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr">
         <is>
           <t>El dashboard debe funcionar como el centro de acompañamiento de Amy. Además de mostrar números, debe traducir el plan financiero en acciones concretas, simples y priorizadas para que la usuaria sepa qué hacer en Finance BFF y en su vida real.</t>
         </is>
       </c>
-      <c r="F14" s="5" t="inlineStr">
+      <c r="F14" s="6" t="inlineStr">
         <is>
           <t>Como una mujer que acaba de terminar de organizar sus finanzas con Amy, quiero que al llegar a Mis finanzas me expliquen qué construimos juntas y cuáles son mis próximos pasos, para no sentir que después del onboarding quedé sola frente a un dashboard.</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr">
+      <c r="G14" s="6" t="inlineStr">
         <is>
           <t>Incorporar en Mis finanzas un bloque visible de acompañamiento, por ejemplo 'Tu plan con Amy' o 'Qué hacer ahora'. Mostrar pocas acciones prioritarias según el escenario de la usuaria, con CTA directo al módulo correspondiente. En el Happy Path pueden incluir: preparar cajitas en el banco, crear bolsitas de ahorro, registrar gastos de la semana y completar las transferencias recomendadas.</t>
         </is>
       </c>
-      <c r="H14" s="5" t="inlineStr">
+      <c r="H14" s="6" t="inlineStr">
         <is>
           <t>El dashboard no debe convertirse en una lista pesada de pendientes. Priorizar máximo las acciones que realmente requieren atención y marcar visualmente las completadas. Amy debe mantener el tono de acompañamiento del onboarding.</t>
         </is>
       </c>
-      <c r="I14" s="5" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>Transformar Finance BFF de una herramienta de visualización en una experiencia de acompañamiento financiero continuo.</t>
         </is>
       </c>
-      <c r="J14" s="5" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr">
         <is>
           <t>La usuaria entra al dashboard y sabe inmediatamente qué debe hacer después.</t>
         </is>
       </c>
-      <c r="K14" s="5" t="inlineStr">
+      <c r="K14" s="6" t="inlineStr">
         <is>
           <t>El dashboard presenta próximos pasos accionables y cada acción lleva directamente al lugar donde puede completarse o aprender cómo hacerla.</t>
         </is>
       </c>
-      <c r="L14" s="5" t="inlineStr">
+      <c r="L14" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="M14" s="5" t="inlineStr">
+      <c r="M14" s="6" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="120" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+    <row r="15" ht="76.8" customFormat="1" customHeight="1" s="8">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Hábitos financieros y conexión con el banco</t>
         </is>
@@ -1380,64 +1414,64 @@
           <t>3.7</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Guiar la creación de cajitas y bolsitas en el banco</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Finance BFF calcula cuánto reservar para cajitas y bolsitas, pero la aplicación no mueve físicamente el dinero. En algunos puntos se explica parcialmente qué hacer en el banco, mientras que en otros esta conexión con la vida real no es suficientemente visible.</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>La usuaria debe entender que Finance BFF organiza el plan y que ella debe separar el dinero en su banco. Amy debe convertir cada recomendación en una instrucción sencilla y permitir registrar que la acción ya fue realizada.</t>
         </is>
       </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>Como una mujer que ya definió sus cajitas y bolsitas con Amy, quiero saber exactamente qué debo hacer en mi banco con esos montos, para que mi organización en Finance BFF se convierta en dinero realmente separado y no se quede solo en un plan dentro de la aplicación.</t>
         </is>
       </c>
-      <c r="G15" s="5" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
         <is>
           <t>En Cajitas y Bolsitas de ahorro incluir instrucciones visibles sobre la acción bancaria correspondiente. Indicar qué monto total separar y, cuando aplique, cuánto corresponde a cada cajita o bolsita. Permitir marcar la transferencia mensual como realizada. Desde Mis finanzas, enlazar las tareas pendientes directamente a estos módulos.</t>
         </is>
       </c>
-      <c r="H15" s="5" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Evitar dar la impresión de que Finance BFF ya movió el dinero. Diferenciar claramente entre 'Amy reserva en tu presupuesto' y 'tú separas/transfieres en tu banco'. Usar lenguaje sencillo y accionable.</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>Conectar la planificación digital con comportamientos financieros reales y aumentar la efectividad del producto.</t>
         </is>
       </c>
-      <c r="J15" s="5" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>La usuaria entiende qué debe separar en su banco, lo hace y puede reflejar la acción en Finance BFF.</t>
         </is>
       </c>
-      <c r="K15" s="5" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>Los módulos explican explícitamente la acción bancaria y permiten registrar el cumplimiento mensual sin confundir reserva presupuestal con transferencia real.</t>
         </is>
       </c>
-      <c r="L15" s="5" t="inlineStr">
+      <c r="L15" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="M15" s="5" t="inlineStr">
+      <c r="M15" s="6" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="120" customHeight="1">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="16" ht="76.8" customFormat="1" customHeight="1" s="8">
+      <c r="A16" s="6" t="inlineStr">
         <is>
           <t>Hábitos financieros y conexión con el banco</t>
         </is>
@@ -1447,64 +1481,64 @@
           <t>3.8</t>
         </is>
       </c>
-      <c r="C16" s="5" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
         <is>
           <t>Crear el ritual semanal de registro de gastos</t>
         </is>
       </c>
-      <c r="D16" s="5" t="inlineStr">
+      <c r="D16" s="6" t="inlineStr">
         <is>
           <t>Mis gastos permite registrar transacciones manualmente o hablando con Amy, pero actualmente la funcionalidad depende de que la usuaria recuerde entrar por iniciativa propia.</t>
         </is>
       </c>
-      <c r="E16" s="5" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>Finance BFF debe ayudar a convertir el registro de gastos en un hábito simple y sostenible. Amy debe proponer una rutina semanal corta para revisar y registrar los gastos de los últimos días.</t>
         </is>
       </c>
-      <c r="F16" s="5" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>Como una mujer que quiere tener una mejor relación con su dinero pero no quiere estar pendiente de cada compra todos los días, quiero tener un momento semanal sencillo para contarle a Amy en qué gasté, para mantener mis finanzas actualizadas sin sentir que llevar control es una carga.</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>Presentar en Mis gastos una rutina recomendada de actualización semanal. Explicar que puede dedicar unos minutos una vez por semana, idealmente domingo o lunes, a registrar los gastos de la semana usando voz o ingreso manual. Integrar esta acción dentro del plan del dashboard y permitir identificar cuándo la semana ya fue actualizada.</t>
         </is>
       </c>
-      <c r="H16" s="5" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>El hábito debe sentirse liviano y realista. No transmitir culpa si la usuaria se atrasa. La voz debe presentarse como la forma más fácil de ponerse al día, no como una obligación.</t>
         </is>
       </c>
-      <c r="I16" s="5" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>Incrementar la recurrencia de uso y ayudar a construir hábitos financieros sostenibles.</t>
         </is>
       </c>
-      <c r="J16" s="5" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>La usuaria comprende cuándo y cómo actualizar sus gastos y percibe el proceso como un pequeño ritual semanal.</t>
         </is>
       </c>
-      <c r="K16" s="5" t="inlineStr">
+      <c r="K16" s="6" t="inlineStr">
         <is>
           <t>Mis gastos comunica la rutina semanal y el dashboard puede reflejar si la actualización de la semana está pendiente o completada.</t>
         </is>
       </c>
-      <c r="L16" s="5" t="inlineStr">
+      <c r="L16" s="6" t="inlineStr">
         <is>
           <t>Alta</t>
         </is>
       </c>
-      <c r="M16" s="5" t="inlineStr">
+      <c r="M16" s="6" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="120" customHeight="1">
-      <c r="A17" s="5" t="inlineStr">
+    <row r="17" ht="76.8" customFormat="1" customHeight="1" s="8">
+      <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Acompañamiento después del onboarding</t>
         </is>
@@ -1514,57 +1548,1196 @@
           <t>3.9</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>Enseñar cómo usar el menú principal</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>Después del onboarding aparecen varios módulos en el menú lateral, pero una usuaria nueva puede no saber qué función cumple cada uno ni cuándo debería entrar a cada sección.</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>La primera llegada al dashboard debe orientar brevemente sobre la estructura de Finance BFF y mostrar que el menú lateral es el lugar desde donde administrará cada parte de su vida financiera.</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>Como una mujer que acaba de terminar el onboarding y ve por primera vez Mis finanzas, Mis gastos, Cajitas, Bolsitas de ahorro y Deudas, quiero entender para qué sirve cada sección y cuándo debo usarla, para moverme con seguridad sin tener que descubrir sola cómo funciona la plataforma.</t>
         </is>
       </c>
-      <c r="G17" s="5" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
         <is>
           <t>Incluir una guía inicial breve en la primera entrada al dashboard que presente el menú lateral y explique el propósito de cada módulo en una frase. Evitar un tour largo. Permitir omitirlo y no repetirlo automáticamente después de completarlo.</t>
         </is>
       </c>
-      <c r="H17" s="5" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>La orientación debe ser contextual y ligera. No bloquear innecesariamente el uso del dashboard ni convertir la primera entrada en otro onboarding extenso.</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>Reducir confusión inicial y acelerar la adopción de los módulos principales.</t>
         </is>
       </c>
-      <c r="J17" s="5" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>La usuaria entiende dónde registrar gastos, gestionar cajitas, organizar ahorro y revisar deudas.</t>
         </is>
       </c>
-      <c r="K17" s="5" t="inlineStr">
+      <c r="K17" s="6" t="inlineStr">
         <is>
           <t>La guía aparece en la primera entrada, puede omitirse y no vuelve a mostrarse una vez completada.</t>
         </is>
       </c>
-      <c r="L17" s="5" t="inlineStr">
+      <c r="L17" s="6" t="inlineStr">
         <is>
           <t>Media</t>
         </is>
       </c>
-      <c r="M17" s="5" t="inlineStr">
+      <c r="M17" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="99.3" customHeight="1">
+      <c r="A18" s="9" t="inlineStr">
+        <is>
+          <t>Onboarding Happy Path</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>3.10</t>
+        </is>
+      </c>
+      <c r="C18" s="9" t="inlineStr">
+        <is>
+          <t>Simplificar la selección de país</t>
+        </is>
+      </c>
+      <c r="D18" s="9" t="inlineStr">
+        <is>
+          <t>El paso de país presenta demasiado texto y puede resultar abrumador.</t>
+        </is>
+      </c>
+      <c r="E18" s="9" t="inlineStr">
+        <is>
+          <t>Seleccionar el país de forma rápida mediante una lista desplegable con búsqueda.</t>
+        </is>
+      </c>
+      <c r="F18" s="9" t="inlineStr">
+        <is>
+          <t>Como una usuaria que está comenzando su configuración, quiero encontrar mi país sin leer una lista extensa, para continuar rápidamente.</t>
+        </is>
+      </c>
+      <c r="G18" s="9" t="inlineStr">
+        <is>
+          <t>Reemplazar la presentación extensa por un selector desplegable con búsqueda por nombre. Permitir escribir para filtrar países y seleccionar una opción válida. Conservar la selección al regresar.</t>
+        </is>
+      </c>
+      <c r="H18" s="9" t="inlineStr">
+        <is>
+          <t>Mostrar una instrucción breve y evitar sobrecargar la pantalla.</t>
+        </is>
+      </c>
+      <c r="I18" s="9" t="inlineStr">
+        <is>
+          <t>Reducir fricción en el registro.</t>
+        </is>
+      </c>
+      <c r="J18" s="9" t="inlineStr">
+        <is>
+          <t>La usuaria encuentra y selecciona su país fácilmente.</t>
+        </is>
+      </c>
+      <c r="K18" s="9" t="inlineStr">
+        <is>
+          <t>Se puede buscar, seleccionar y conservar un país válido.</t>
+        </is>
+      </c>
+      <c r="L18" s="9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="M18" s="9" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="99.3" customHeight="1">
+      <c r="A19" s="9" t="inlineStr">
+        <is>
+          <t>Onboarding Happy Path</t>
+        </is>
+      </c>
+      <c r="B19" s="10" t="inlineStr">
+        <is>
+          <t>3.11</t>
+        </is>
+      </c>
+      <c r="C19" s="9" t="inlineStr">
+        <is>
+          <t>Permitir configurar varias monedas</t>
+        </is>
+      </c>
+      <c r="D19" s="9" t="inlineStr">
+        <is>
+          <t>El paso de moneda permite seleccionar una sola moneda, aunque la usuaria puede manejar dinero en varias.</t>
+        </is>
+      </c>
+      <c r="E19" s="9" t="inlineStr">
+        <is>
+          <t>Permitir registrar una moneda principal y otras monedas utilizadas.</t>
+        </is>
+      </c>
+      <c r="F19" s="9" t="inlineStr">
+        <is>
+          <t>Como una usuaria que recibe, gasta o ahorra dinero en distintas monedas, quiero configurar todas las que utilizo, para representar mi realidad financiera sin limitarme a una sola.</t>
+        </is>
+      </c>
+      <c r="G19" s="9" t="inlineStr">
+        <is>
+          <t>Permitir seleccionar varias monedas y distinguir una principal. Conservar la configuración para los registros posteriores. Definir cómo se mostrarán los montos por moneda y evitar sumarlos directamente sin una conversión explícita.</t>
+        </is>
+      </c>
+      <c r="H19" s="9" t="inlineStr">
+        <is>
+          <t>No asumir que todos los valores comparten moneda. La configuración debe seguir siendo sencilla para quien utiliza solo una.</t>
+        </is>
+      </c>
+      <c r="I19" s="9" t="inlineStr">
+        <is>
+          <t>Representar situaciones financieras reales y evitar cálculos engañosos.</t>
+        </is>
+      </c>
+      <c r="J19" s="9" t="inlineStr">
+        <is>
+          <t>La usuaria puede configurar sus monedas y reconocer la moneda de cada monto.</t>
+        </is>
+      </c>
+      <c r="K19" s="9" t="inlineStr">
+        <is>
+          <t>Se pueden guardar varias monedas y una principal; los totales no mezclan monedas sin conversión definida.</t>
+        </is>
+      </c>
+      <c r="L19" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M19" s="9" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="99.3" customHeight="1">
+      <c r="A20" s="9" t="inlineStr">
+        <is>
+          <t>Onboarding Happy Path</t>
+        </is>
+      </c>
+      <c r="B20" s="10" t="inlineStr">
+        <is>
+          <t>3.12</t>
+        </is>
+      </c>
+      <c r="C20" s="9" t="inlineStr">
+        <is>
+          <t>Eliminar guiones -Hyphens innecesarios de los textos</t>
+        </is>
+      </c>
+      <c r="D20" s="9" t="inlineStr">
+        <is>
+          <t>Persisten guiones - hyphens utilizados como recurso de redacción en distintos textos de la experiencia.</t>
+        </is>
+      </c>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Mantener una redacción natural, limpia y consistente con la voz de Finance BFF.</t>
+        </is>
+      </c>
+      <c r="F20" s="9" t="inlineStr">
+        <is>
+          <t>Como una usuaria que interactúa con Amy, quiero leer mensajes fluidos y cercanos, para comprenderlos sin interrupciones visuales innecesarias que se vean generados por AI</t>
+        </is>
+      </c>
+      <c r="G20" s="9" t="inlineStr">
+        <is>
+          <t>Revisar exhaustivamente todos los textos del onboarding y del producto y eliminar los guiones usados como separadores de frases. Reescribir las oraciones cuando sea necesario. Conservar únicamente los guiones que tengan una función legítima, como signos matemáticos o parte de un dato.</t>
+        </is>
+      </c>
+      <c r="H20" s="9" t="inlineStr">
+        <is>
+          <t>No eliminar signos necesarios para cálculos, fechas o información técnica. Evitar sustituciones mecánicas que deterioren la redacción.</t>
+        </is>
+      </c>
+      <c r="I20" s="9" t="inlineStr">
+        <is>
+          <t>Mantener consistencia editorial y calidad percibida.</t>
+        </is>
+      </c>
+      <c r="J20" s="9" t="inlineStr">
+        <is>
+          <t>Los mensajes se sienten naturales y coherentes con la marca.</t>
+        </is>
+      </c>
+      <c r="K20" s="9" t="inlineStr">
+        <is>
+          <t>La revisión editorial no encuentra guiones innecesarios en los textos visibles.</t>
+        </is>
+      </c>
+      <c r="L20" s="9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="M20" s="9" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="99.3" customHeight="1">
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>Onboarding Happy Path</t>
+        </is>
+      </c>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>3.13</t>
+        </is>
+      </c>
+      <c r="C21" s="9" t="inlineStr">
+        <is>
+          <t>Aclarar que los gastos fijos pueden completarse después</t>
+        </is>
+      </c>
+      <c r="D21" s="9" t="inlineStr">
+        <is>
+          <t>Al registrar gastos fijos uno por uno, la usuaria puede sentir que debe recordar absolutamente todos antes de continuar.</t>
+        </is>
+      </c>
+      <c r="E21" s="9" t="inlineStr">
+        <is>
+          <t>Explicar que puede agregar o corregir gastos más adelante sin perder su progreso.</t>
+        </is>
+      </c>
+      <c r="F21" s="9" t="inlineStr">
+        <is>
+          <t>Como una usuaria que está registrando sus gastos mensuales y puede olvidar alguno, quiero saber que podré agregarlo después, para avanzar sin sentir que debo tener toda la información perfecta.</t>
+        </is>
+      </c>
+      <c r="G21" s="9" t="inlineStr">
+        <is>
+          <t>Agregar una nota breve junto al formulario de gastos fijos indicando que podrá añadir o editar gastos posteriormente desde la aplicación. Mantener el acceso a la edición después del onboarding.</t>
+        </is>
+      </c>
+      <c r="H21" s="9" t="inlineStr">
+        <is>
+          <t>El mensaje debe dar tranquilidad sin restar importancia a registrar información lo más completa posible.</t>
+        </is>
+      </c>
+      <c r="I21" s="9" t="inlineStr">
+        <is>
+          <t>Reducir abandono y facilitar la actualización de datos.</t>
+        </is>
+      </c>
+      <c r="J21" s="9" t="inlineStr">
+        <is>
+          <t>La usuaria continúa con confianza y sabe que puede completar sus gastos después.</t>
+        </is>
+      </c>
+      <c r="K21" s="9" t="inlineStr">
+        <is>
+          <t>La nota es visible y existe una ruta funcional para agregar o editar gastos posteriormente.</t>
+        </is>
+      </c>
+      <c r="L21" s="9" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="M21" s="9" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="99.3" customHeight="1">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>Onboarding Happy Path</t>
+        </is>
+      </c>
+      <c r="B22" s="10" t="inlineStr">
+        <is>
+          <t>3.14</t>
+        </is>
+      </c>
+      <c r="C22" s="9" t="inlineStr">
+        <is>
+          <t>Proponer la próxima fecha válida para cajitas</t>
+        </is>
+      </c>
+      <c r="D22" s="9" t="inlineStr">
+        <is>
+          <t>Al crear una cajita, el selector puede permitir una fecha de pago que ya pasó, como junio de 2026 cuando se está configurando en septiembre de 2026.</t>
+        </is>
+      </c>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>Proponer automáticamente la próxima fecha futura correspondiente al gasto.</t>
+        </is>
+      </c>
+      <c r="F22" s="9" t="inlineStr">
+        <is>
+          <t>Como una usuaria que está preparando gastos que se repiten, quiero que Amy me sugiera la próxima fecha de pago válida, para no crear una cajita con una fecha vencida.</t>
+        </is>
+      </c>
+      <c r="G22" s="9" t="inlineStr">
+        <is>
+          <t>Al seleccionar un mes o fecha de vencimiento, calcular la próxima ocurrencia futura según la periodicidad del gasto y la fecha actual. Si el gasto es anual y junio de este año ya pasó, proponer junio del año siguiente. Permitir ajustar la fecha y recalcular la reserva correspondiente.</t>
+        </is>
+      </c>
+      <c r="H22" s="9" t="inlineStr">
+        <is>
+          <t>No asumir que todos los gastos son anuales. Mostrar claramente mes y año y evitar fechas pasadas por defecto.</t>
+        </is>
+      </c>
+      <c r="I22" s="9" t="inlineStr">
+        <is>
+          <t>Evitar errores de planificación y mejorar la precisión de las reservas.</t>
+        </is>
+      </c>
+      <c r="J22" s="9" t="inlineStr">
+        <is>
+          <t>La cajita se configura con una fecha futura coherente con su periodicidad.</t>
+        </is>
+      </c>
+      <c r="K22" s="9" t="inlineStr">
+        <is>
+          <t>Un gasto anual cuyo mes ya pasó propone el año siguiente y recalcula correctamente su reserva.</t>
+        </is>
+      </c>
+      <c r="L22" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M22" s="9" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="99.3" customHeight="1">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t>Onboarding Happy Path</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>3.15</t>
+        </is>
+      </c>
+      <c r="C23" s="9" t="inlineStr">
+        <is>
+          <t>Calcular la recomendación después de definir importancia en la creación de bolsitas de ahorro</t>
+        </is>
+      </c>
+      <c r="D23" s="9" t="inlineStr">
+        <is>
+          <t>La recomendación de Amy aparece antes de que la usuaria seleccione la importancia de la bolsita.</t>
+        </is>
+      </c>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>Primero conocer la prioridad de la usuaria y después calcular una recomendación personalizada.</t>
+        </is>
+      </c>
+      <c r="F23" s="9" t="inlineStr">
+        <is>
+          <t>Como una usuaria que está creando una bolsita de ahorro, quiero indicar qué tan importante es para mí antes de recibir una recomendación, para sentir que Amy tiene en cuenta mis prioridades.</t>
+        </is>
+      </c>
+      <c r="G23" s="9" t="inlineStr">
+        <is>
+          <t>Ubicar las estrellas de importancia antes del bloque de recomendación. Inicializar el monto recomendado en $0 hasta que se seleccione una importancia. Recalcular la recomendación cuando cambie la prioridad y permitir aceptar o editar el monto.</t>
+        </is>
+      </c>
+      <c r="H23" s="9" t="inlineStr">
+        <is>
+          <t>No presentar una recomendación como personalizada antes de contar con la información necesaria. Explicar brevemente que la importancia ayuda a Amy a proponer un monto.</t>
+        </is>
+      </c>
+      <c r="I23" s="9" t="inlineStr">
+        <is>
+          <t>Mejorar la relevancia y confianza en las recomendaciones.</t>
+        </is>
+      </c>
+      <c r="J23" s="9" t="inlineStr">
+        <is>
+          <t>La usuaria entiende que su prioridad influye en el monto sugerido.</t>
+        </is>
+      </c>
+      <c r="K23" s="9" t="inlineStr">
+        <is>
+          <t>La recomendación inicia en $0, se calcula después de seleccionar importancia y se actualiza al cambiarla.</t>
+        </is>
+      </c>
+      <c r="L23" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M23" s="9" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="99.3" customHeight="1">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
+          <t>Onboarding Happy Path</t>
+        </is>
+      </c>
+      <c r="B24" s="10" t="inlineStr">
+        <is>
+          <t>3.16</t>
+        </is>
+      </c>
+      <c r="C24" s="9" t="inlineStr">
+        <is>
+          <t>Hacer evidente la acción Agregar bolsita</t>
+        </is>
+      </c>
+      <c r="D24" s="9" t="inlineStr">
+        <is>
+          <t>Después de seleccionar o editar el monto, no resulta suficientemente claro que debe pulsarse Agregar bolsita para incorporarla al reparto.</t>
+        </is>
+      </c>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>La acción de agregar debe destacarse y dejar claro cuándo el monto ya forma parte del ahorro distribuido.</t>
+        </is>
+      </c>
+      <c r="F24" s="9" t="inlineStr">
+        <is>
+          <t>Como una usuaria que está creando sus bolsitas, quiero identificar fácilmente cómo confirmar cada una, para saber que quedó agregada y que el dinero restante se actualizó.</t>
+        </is>
+      </c>
+      <c r="G24" s="9" t="inlineStr">
+        <is>
+          <t>Dar mayor jerarquía visual al botón Agregar bolsita cuando los datos estén completos. Utilizar un estado de color claramente diferenciado dentro de la paleta de marca. Al agregar, mostrar la bolsita en la lista y actualizar inmediatamente los totales.</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="inlineStr">
+        <is>
+          <t>Distinguir visualmente entre editar o aceptar una recomendación y confirmar la creación de la bolsita. No depender únicamente del color para comunicar el estado.</t>
+        </is>
+      </c>
+      <c r="I24" s="9" t="inlineStr">
+        <is>
+          <t>Reducir errores y facilitar la finalización del reparto.</t>
+        </is>
+      </c>
+      <c r="J24" s="9" t="inlineStr">
+        <is>
+          <t>La usuaria identifica la acción de confirmación y ve el resultado inmediatamente.</t>
+        </is>
+      </c>
+      <c r="K24" s="9" t="inlineStr">
+        <is>
+          <t>El botón se distingue claramente y al pulsarlo se agrega la bolsita y se actualiza el saldo.</t>
+        </is>
+      </c>
+      <c r="L24" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M24" s="9" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="99.3" customHeight="1">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>Onboarding Happy Path</t>
+        </is>
+      </c>
+      <c r="B25" s="10" t="inlineStr">
+        <is>
+          <t>3.17</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Mantener visible el resumen del reparto de ahorro</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Al agregar varias bolsitas, el resumen de dinero repartido y restante se desplaza hacia arriba y deja de estar visible.</t>
+        </is>
+      </c>
+      <c r="E25" s="9" t="inlineStr">
+        <is>
+          <t>Mantener siempre a la vista cuánto ahorro mensual se ha asignado y cuánto queda disponible.</t>
+        </is>
+      </c>
+      <c r="F25" s="9" t="inlineStr">
+        <is>
+          <t>Como una usuaria que está distribuyendo su ahorro entre varias bolsitas, quiero consultar el total asignado y el saldo restante sin tener que desplazarme hacia arriba, para tomar decisiones con claridad mientras agrego nuevas bolsitas.</t>
+        </is>
+      </c>
+      <c r="G25" s="9" t="inlineStr">
+        <is>
+          <t>Implementar un resumen persistente o sticky que muestre ahorro mensual total, monto ya repartido y saldo restante. Actualizarlo al agregar, editar o eliminar bolsitas. Adaptar su ubicación a desktop y móvil sin tapar campos ni acciones.</t>
+        </is>
+      </c>
+      <c r="H25" s="9" t="inlineStr">
+        <is>
+          <t>El resumen debe ser compacto, legible y mantenerse visible durante la interacción. Conservar el estado positivo cuando el reparto llegue a $0.</t>
+        </is>
+      </c>
+      <c r="I25" s="9" t="inlineStr">
+        <is>
+          <t>Mejorar el control del presupuesto y reducir fricción durante la creación.</t>
+        </is>
+      </c>
+      <c r="J25" s="9" t="inlineStr">
+        <is>
+          <t>La usuaria conoce el estado del reparto en todo momento.</t>
+        </is>
+      </c>
+      <c r="K25" s="9" t="inlineStr">
+        <is>
+          <t>El resumen permanece visible durante el desplazamiento y sus tres valores se actualizan correctamente.</t>
+        </is>
+      </c>
+      <c r="L25" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M25" s="9" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="99.3" customHeight="1">
+      <c r="A26" s="9" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>4.1</t>
+        </is>
+      </c>
+      <c r="C26" s="9" t="inlineStr">
+        <is>
+          <t>Confirmar transferencias de cada cajita por separado</t>
+        </is>
+      </c>
+      <c r="D26" s="9" t="inlineStr">
+        <is>
+          <t>El dashboard permite marcar como realizada la transferencia mensual del total de cajitas, pero no distinguir cuáles se han financiado realmente.</t>
+        </is>
+      </c>
+      <c r="E26" s="9" t="inlineStr">
+        <is>
+          <t>Permitir registrar el cumplimiento de cada cajita individualmente y mostrar el avance del mes.</t>
+        </is>
+      </c>
+      <c r="F26" s="9" t="inlineStr">
+        <is>
+          <t>Como una usuaria que separa dinero para diferentes gastos en su banco, quiero marcar cada cajita cuando realice su transferencia, para llevar un control real de cuáles ya financié y cuáles siguen pendientes.</t>
+        </is>
+      </c>
+      <c r="G26" s="9" t="inlineStr">
+        <is>
+          <t>Agregar un check individual de transferencia mensual a cada cajita. Mostrar su monto recomendado y estado del mes. Mantener un resumen del total completado y pendiente. Permitir corregir una confirmación accidental y conservar el historial por mes.</t>
+        </is>
+      </c>
+      <c r="H26" s="9" t="inlineStr">
+        <is>
+          <t>El check debe representar una acción real de la usuaria, no una transferencia ejecutada por Amy. Evitar que confirmar una cajita marque automáticamente las demás.</t>
+        </is>
+      </c>
+      <c r="I26" s="9" t="inlineStr">
+        <is>
+          <t>Facilitar el seguimiento de reservas y reforzar el hábito de separar dinero.</t>
+        </is>
+      </c>
+      <c r="J26" s="9" t="inlineStr">
+        <is>
+          <t>La usuaria sabe qué cajitas ya financió y cuáles faltan.</t>
+        </is>
+      </c>
+      <c r="K26" s="9" t="inlineStr">
+        <is>
+          <t>Cada cajita puede confirmarse independientemente y el resumen refleja únicamente las confirmaciones correspondientes.</t>
+        </is>
+      </c>
+      <c r="L26" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M26" s="9" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="99.3" customHeight="1">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="B27" s="10" t="inlineStr">
+        <is>
+          <t>4.2</t>
+        </is>
+      </c>
+      <c r="C27" s="9" t="inlineStr">
+        <is>
+          <t>Guiar y confirmar los abonos de cada bolsita</t>
+        </is>
+      </c>
+      <c r="D27" s="9" t="inlineStr">
+        <is>
+          <t>El módulo de bolsitas muestra el plan de ahorro, pero no explica suficientemente que el dinero debe separarse en el banco ni permite registrar claramente el cumplimiento de cada aporte mensual.</t>
+        </is>
+      </c>
+      <c r="E27" s="9" t="inlineStr">
+        <is>
+          <t>Conectar cada bolsita con una acción bancaria concreta y permitir confirmar sus aportes.</t>
+        </is>
+      </c>
+      <c r="F27" s="9" t="inlineStr">
+        <is>
+          <t>Como una usuaria que ya creó sus bolsitas de ahorro, quiero saber cuánto debo separar en mi banco y marcar cada aporte cuando lo realice, para convertir mi plan en un hábito y mantener un seguimiento confiable.</t>
+        </is>
+      </c>
+      <c r="G27" s="9" t="inlineStr">
+        <is>
+          <t>Incluir instrucciones visibles para crear o utilizar bolsillos, sobres o cuentas de ahorro en el banco. Mostrar el aporte mensual de cada bolsita y permitir marcarlo como realizado individualmente. Conservar el estado por mes y permitir corregir confirmaciones. Vincular las acciones pendientes con el dashboard principal.</t>
+        </is>
+      </c>
+      <c r="H27" s="9" t="inlineStr">
+        <is>
+          <t>Diferenciar claramente entre el monto planeado, el dinero efectivamente ahorrado y una transferencia confirmada. No afirmar que Amy mueve dinero automáticamente.</t>
+        </is>
+      </c>
+      <c r="I27" s="9" t="inlineStr">
+        <is>
+          <t>Promover hábitos de ahorro y conectar la planificación con acciones reales.</t>
+        </is>
+      </c>
+      <c r="J27" s="9" t="inlineStr">
+        <is>
+          <t>La usuaria sabe qué hacer en su banco y puede registrar cada aporte realizado.</t>
+        </is>
+      </c>
+      <c r="K27" s="9" t="inlineStr">
+        <is>
+          <t>Cada bolsita permite confirmar su aporte mensual y muestra correctamente su estado pendiente o completado.</t>
+        </is>
+      </c>
+      <c r="L27" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M27" s="9" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="99.3" customHeight="1">
+      <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>4.3</t>
+        </is>
+      </c>
+      <c r="C28" s="9" t="inlineStr">
+        <is>
+          <t>Actualizar el saldo disponible al confirmar movimientos</t>
+        </is>
+      </c>
+      <c r="D28" s="9" t="inlineStr">
+        <is>
+          <t>Al marcar como realizados los aportes de cajitas o bolsitas, el dinero disponible del dashboard en la página principal no se actualiza de forma coherente.</t>
+        </is>
+      </c>
+      <c r="E28" s="9" t="inlineStr">
+        <is>
+          <t>El saldo debe reflejar los movimientos reales confirmados sin descontar dos veces el dinero que ya estaba reservado en el presupuesto.</t>
+        </is>
+      </c>
+      <c r="F28" s="9" t="inlineStr">
+        <is>
+          <t>Como una usuaria que confirma que ya separó dinero para sus cajitas o bolsitas, quiero que el dashboard refleje correctamente ese movimiento, para confiar en el saldo disponible y saber cuánto puedo gastar realmente.</t>
+        </is>
+      </c>
+      <c r="G28" s="9" t="inlineStr">
+        <is>
+          <t>Revisar y corregir la lógica de actualización del saldo disponible al confirmar, editar o revertir aportes. Definir de forma explícita la diferencia entre saldo presupuestado, dinero reservado y dinero efectivamente transferido. Si las reservas ya fueron descontadas al calcular el disponible, una confirmación no debe volver a descontarlas. Mantener consistencia entre dashboard y módulos.</t>
+        </is>
+      </c>
+      <c r="H28" s="9" t="inlineStr">
+        <is>
+          <t>Mostrar con claridad qué representa cada saldo. Evitar cambios inesperados y explicar el efecto de una confirmación cuando corresponda.</t>
+        </is>
+      </c>
+      <c r="I28" s="9" t="inlineStr">
+        <is>
+          <t>Garantizar confianza en los cálculos y evitar decisiones basadas en saldos incorrectos.</t>
+        </is>
+      </c>
+      <c r="J28" s="9" t="inlineStr">
+        <is>
+          <t>El dashboard y los módulos muestran cifras coherentes con el presupuesto y los movimientos confirmados.</t>
+        </is>
+      </c>
+      <c r="K28" s="9" t="inlineStr">
+        <is>
+          <t>Confirmar o revertir un aporte actualiza los estados y saldos correspondientes sin duplicar descuentos ni alterar indebidamente el disponible.</t>
+        </is>
+      </c>
+      <c r="L28" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M28" s="9" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="99.3" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Dashboard</t>
+        </is>
+      </c>
+      <c r="B29" s="10" t="inlineStr">
+        <is>
+          <t>4.4</t>
+        </is>
+      </c>
+      <c r="C29" s="9" t="inlineStr">
+        <is>
+          <t>Registrar el pago de gastos fijos y reflejarlo en el saldo</t>
+        </is>
+      </c>
+      <c r="D29" s="9" t="inlineStr">
+        <is>
+          <t>Mis gastos muestra los gastos fijos registrados, pero no permite identificar fácilmente cuáles ya fueron pagados durante el mes ni refleja ese seguimiento en el dashboard principal.</t>
+        </is>
+      </c>
+      <c r="E29" s="9" t="inlineStr">
+        <is>
+          <t>Permitir marcar cada gasto fijo como pagado y mantener un saldo disponible coherente con los pagos y compromisos del mes.</t>
+        </is>
+      </c>
+      <c r="F29" s="9" t="inlineStr">
+        <is>
+          <t>Como una usuaria que paga sus gastos fijos en diferentes momentos del mes, quiero marcar cada uno cuando lo pague y ver cuáles siguen pendientes, para organizar mis pagos y conocer cuánto dinero tengo realmente disponible.</t>
+        </is>
+      </c>
+      <c r="G29" s="9" t="inlineStr">
+        <is>
+          <t>Agregar un check individual de pago a cada gasto fijo en Mis gastos. Mostrar estado pagado o pendiente por mes y permitir corregirlo. Reflejar el cumplimiento en Mis finanzas y actualizar los saldos pertinentes. Definir la lógica para que un gasto fijo ya descontado del presupuesto no vuelva a descontarse al marcarlo como pagado.</t>
+        </is>
+      </c>
+      <c r="H29" s="9" t="inlineStr">
+        <is>
+          <t>Distinguir entre gasto presupuestado y pago realizado. Mantener visibles los pendientes sin presentar un gasto pagado como una nueva salida adicional de dinero.</t>
+        </is>
+      </c>
+      <c r="I29" s="9" t="inlineStr">
+        <is>
+          <t>Facilitar el control de pagos y mejorar la confiabilidad del dashboard.</t>
+        </is>
+      </c>
+      <c r="J29" s="9" t="inlineStr">
+        <is>
+          <t>La usuaria identifica qué gastos ya pagó y cuánto dinero queda disponible sin duplicaciones.</t>
+        </is>
+      </c>
+      <c r="K29" s="9" t="inlineStr">
+        <is>
+          <t>Cada gasto fijo puede marcarse individualmente y el dashboard refleja el estado y los saldos correctos sin doble descuento.</t>
+        </is>
+      </c>
+      <c r="L29" s="9" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M29" s="9" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="139.95" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
+        <is>
+          <t>Dashboard | Mis deudas</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="inlineStr">
+        <is>
+          <t>4.5</t>
+        </is>
+      </c>
+      <c r="C30" s="11" t="inlineStr">
+        <is>
+          <t>Convertir la metodología de deuda en un plan de acción mensual</t>
+        </is>
+      </c>
+      <c r="D30" s="11" t="inlineStr">
+        <is>
+          <t>El módulo Mis deudas muestra la metodología recomendada, el orden sugerido y los saldos de las deudas, pero la usuaria todavía tiene que interpretar por sí sola qué debería hacer durante el mes. La información explica el enfoque, pero no termina de traducirlo en acciones concretas y priorizadas.</t>
+        </is>
+      </c>
+      <c r="E30" s="11" t="inlineStr">
+        <is>
+          <t>Al entrar a Mis deudas, la usuaria debe recibir un plan simple y accionable para ese mes. Amy debe indicarle qué pagos mínimos o cuotas debe cubrir en todas sus deudas, cuál es la deuda prioritaria según la metodología elegida y qué hacer si tiene dinero adicional disponible para acelerar su progreso.</t>
+        </is>
+      </c>
+      <c r="F30" s="11" t="inlineStr">
+        <is>
+          <t>Como una mujer que tiene más de una deuda y ya recibió una metodología personalizada de Amy, quiero saber exactamente qué debo hacer este mes con cada deuda, para aplicar la estrategia sin tener que interpretar sola cómo funciona.</t>
+        </is>
+      </c>
+      <c r="G30" s="11" t="inlineStr">
+        <is>
+          <t>Incorporar un bloque visible llamado, por ejemplo, 'Tu plan de este mes'. Debe listar primero las obligaciones que deben mantenerse al día y después destacar la deuda prioritaria según el método seleccionado. Si existe capacidad para un pago adicional, explicar que ese dinero debe dirigirse a la deuda prioritaria. Cada acción debe enlazar con el registro del pago correspondiente. El plan debe actualizarse cuando cambien los saldos, se agregue una deuda o una deuda se liquide.</t>
+        </is>
+      </c>
+      <c r="H30" s="11" t="inlineStr">
+        <is>
+          <t>El lenguaje debe ser directo, corto y orientado a la acción. Evitar repetir una explicación extensa de la metodología. La usuaria ya sabe qué método tiene; aquí necesita saber qué hacer ahora. Diferenciar visualmente 'mantener al día' de 'acelerar esta deuda'.</t>
+        </is>
+      </c>
+      <c r="I30" s="11" t="inlineStr">
+        <is>
+          <t>Convertir la metodología elegida en comportamiento financiero real y aumentar la utilidad recurrente de Amy.</t>
+        </is>
+      </c>
+      <c r="J30" s="11" t="inlineStr">
+        <is>
+          <t>La usuaria entiende qué debe pagar, qué deuda tiene prioridad y dónde dirigir cualquier dinero adicional.</t>
+        </is>
+      </c>
+      <c r="K30" s="11" t="inlineStr">
+        <is>
+          <t>Al entrar a Mis deudas existe un plan mensual claro, alineado con la metodología guardada, y las acciones cambian correctamente cuando cambian los datos de deuda.</t>
+        </is>
+      </c>
+      <c r="L30" s="11" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M30" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="139.95" customHeight="1">
+      <c r="A31" s="11" t="inlineStr">
+        <is>
+          <t>Dashboard | Mis deudas</t>
+        </is>
+      </c>
+      <c r="B31" s="12" t="inlineStr">
+        <is>
+          <t>4.6</t>
+        </is>
+      </c>
+      <c r="C31" s="11" t="inlineStr">
+        <is>
+          <t>Diferenciar cuota normal y abono adicional a capital</t>
+        </is>
+      </c>
+      <c r="D31" s="11" t="inlineStr">
+        <is>
+          <t>Actualmente la acción 'Registrar pago' no explica claramente si la usuaria está registrando la cuota mensual requerida, un pago adicional para reducir la deuda o ambos. Esto puede generar confusión sobre el efecto real del pago en el saldo.</t>
+        </is>
+      </c>
+      <c r="E31" s="11" t="inlineStr">
+        <is>
+          <t>Al registrar un movimiento, Amy debe ayudar a la usuaria a distinguir entre cumplir con su cuota habitual y realizar un abono adicional dirigido a capital. La explicación debe ser breve y educativa, dejando claro que una cuota normal puede incluir intereses, capital y otros cargos, mientras que un abono adicional a capital busca reducir directamente el saldo sujeto a las condiciones de la entidad financiera.</t>
+        </is>
+      </c>
+      <c r="F31" s="11" t="inlineStr">
+        <is>
+          <t>Como una mujer que quiere avanzar con sus deudas pero no domina los términos financieros, quiero entender la diferencia entre pagar mi cuota y hacer un abono adicional a capital, para saber qué acción estoy registrando y cómo puede impactar mi deuda.</t>
+        </is>
+      </c>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>Al seleccionar Registrar pago, solicitar el tipo de movimiento: 'Pago de mi cuota' o 'Abono adicional a capital'. Incluir una explicación contextual breve para cada opción. No asumir que el valor completo de una cuota reduce el capital. Cuando la usuaria registre un abono a capital, aclarar que debe verificar en su banco o entidad financiera que el pago haya sido aplicado a capital y bajo qué condiciones. Permitir registrar ambos movimientos en el mismo mes.</t>
+        </is>
+      </c>
+      <c r="H31" s="11" t="inlineStr">
+        <is>
+          <t>La educación debe aparecer en el momento de la decisión, no como una clase aparte. Usar lenguaje cotidiano. Evitar prometer una reducción específica de intereses o plazo porque depende de las condiciones del crédito.</t>
+        </is>
+      </c>
+      <c r="I31" s="11" t="inlineStr">
+        <is>
+          <t>Mejorar la educación financiera dentro de la experiencia y reducir registros incorrectos.</t>
+        </is>
+      </c>
+      <c r="J31" s="11" t="inlineStr">
+        <is>
+          <t>La usuaria sabe qué tipo de pago está registrando y comprende que ambos movimientos tienen funciones diferentes.</t>
+        </is>
+      </c>
+      <c r="K31" s="11" t="inlineStr">
+        <is>
+          <t>El flujo obliga a identificar el tipo de pago, muestra la explicación correspondiente y no descuenta automáticamente toda cuota del saldo de capital.</t>
+        </is>
+      </c>
+      <c r="L31" s="11" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M31" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="139.95" customHeight="1">
+      <c r="A32" s="11" t="inlineStr">
+        <is>
+          <t>Dashboard | Mis deudas</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="inlineStr">
+        <is>
+          <t>4.7</t>
+        </is>
+      </c>
+      <c r="C32" s="11" t="inlineStr">
+        <is>
+          <t>Confirmar individualmente los pagos realizados en el banco</t>
+        </is>
+      </c>
+      <c r="D32" s="11" t="inlineStr">
+        <is>
+          <t>El módulo permite registrar pagos, pero no existe una rutina visual suficientemente clara para confirmar qué obligaciones del mes ya fueron pagadas en el banco y cuáles siguen pendientes.</t>
+        </is>
+      </c>
+      <c r="E32" s="11" t="inlineStr">
+        <is>
+          <t>Cada deuda debe funcionar como una tarea mensual. La usuaria debe poder marcar cuando realizó el pago correspondiente en su banco y ver de inmediato qué deudas ya están al día y cuáles todavía requieren atención.</t>
+        </is>
+      </c>
+      <c r="F32" s="11" t="inlineStr">
+        <is>
+          <t>Como una mujer que paga varias deudas en fechas diferentes, quiero marcar cada pago cuando lo haga en mi banco, para saber cuáles obligaciones ya cumplí este mes y cuáles todavía me faltan.</t>
+        </is>
+      </c>
+      <c r="G32" s="11" t="inlineStr">
+        <is>
+          <t>Agregar un check mensual individual por deuda asociado al pago de la cuota. Mostrar estados claros como 'Pendiente este mes' y 'Pago de este mes registrado'. Si la usuaria registra el pago desde el flujo de Registrar pago, actualizar automáticamente el check. Permitir corregir una marcación accidental y conservar el historial mensual.</t>
+        </is>
+      </c>
+      <c r="H32" s="11" t="inlineStr">
+        <is>
+          <t>El check debe representar una confirmación de la usuaria, no una verificación bancaria automática. Evitar que marcar una deuda afecte a las demás. Mostrar el progreso del mes de forma positiva, por ejemplo '1 de 2 pagos del mes listos'.</t>
+        </is>
+      </c>
+      <c r="I32" s="11" t="inlineStr">
+        <is>
+          <t>Crear una rutina mensual de seguimiento y reducir pagos olvidados.</t>
+        </is>
+      </c>
+      <c r="J32" s="11" t="inlineStr">
+        <is>
+          <t>La usuaria puede ver de un vistazo qué pagos ya realizó y qué obligaciones siguen pendientes.</t>
+        </is>
+      </c>
+      <c r="K32" s="11" t="inlineStr">
+        <is>
+          <t>Cada deuda puede marcarse de manera independiente, el estado se conserva por mes y el resumen mensual coincide con los pagos registrados.</t>
+        </is>
+      </c>
+      <c r="L32" s="11" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M32" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="139.95" customHeight="1">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>Dashboard | Mis deudas</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="inlineStr">
+        <is>
+          <t>4.8</t>
+        </is>
+      </c>
+      <c r="C33" s="11" t="inlineStr">
+        <is>
+          <t>Actualizar el saldo real de la deuda después de registrar pagos</t>
+        </is>
+      </c>
+      <c r="D33" s="11" t="inlineStr">
+        <is>
+          <t>El dashboard muestra saldos y meses estimados, pero registrar una cuota no permite saber con certeza cuánto disminuyó realmente el capital. Si Amy asume que todo el pago reduce el saldo, puede mostrar un progreso incorrecto.</t>
+        </is>
+      </c>
+      <c r="E33" s="11" t="inlineStr">
+        <is>
+          <t>Después de registrar pagos, Amy debe mantener un saldo de deuda confiable. Cuando no sea posible conocer automáticamente cuánto del pago se aplicó a capital, la usuaria debe poder actualizar el saldo real tomando como referencia la información de su banco o extracto.</t>
+        </is>
+      </c>
+      <c r="F33" s="11" t="inlineStr">
+        <is>
+          <t>Como una mujer que quiere seguir mi avance de forma confiable, quiero que el saldo de cada deuda refleje lo que realmente debo después de mis pagos, para no tomar decisiones basadas en un cálculo incorrecto.</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>No restar automáticamente el valor completo de una cuota normal al saldo de capital salvo que exista información suficiente para hacerlo correctamente. Permitir que la usuaria actualice el saldo actual de la deuda después de revisar su banco o extracto. Para abonos adicionales a capital confirmados, registrar el movimiento y actualizar el saldo según el dato confirmado por la usuaria. Guardar el historial de saldos para medir progreso.</t>
+        </is>
+      </c>
+      <c r="H33" s="11" t="inlineStr">
+        <is>
+          <t>Explicar de forma sencilla por qué Amy puede pedir el saldo actualizado. Evitar que la usuaria sienta que debe hacer cálculos financieros. El dato principal debe ser '¿Cuánto debes hoy según tu banco?'.</t>
+        </is>
+      </c>
+      <c r="I33" s="11" t="inlineStr">
+        <is>
+          <t>Proteger la confiabilidad de los cálculos y del progreso mostrado en Finance BFF.</t>
+        </is>
+      </c>
+      <c r="J33" s="11" t="inlineStr">
+        <is>
+          <t>Los saldos de deuda representan la situación real de la usuaria y no una reducción estimada incorrectamente.</t>
+        </is>
+      </c>
+      <c r="K33" s="11" t="inlineStr">
+        <is>
+          <t>El saldo no disminuye indebidamente por registrar una cuota; puede actualizarse con el saldo real y el historial conserva los cambios.</t>
+        </is>
+      </c>
+      <c r="L33" s="11" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M33" s="11" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="139.95" customHeight="1">
+      <c r="A34" s="11" t="inlineStr">
+        <is>
+          <t>Dashboard | Mis deudas</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="inlineStr">
+        <is>
+          <t>4.9</t>
+        </is>
+      </c>
+      <c r="C34" s="11" t="inlineStr">
+        <is>
+          <t>Mostrar progreso y siguiente objetivo de salida de deudas</t>
+        </is>
+      </c>
+      <c r="D34" s="11" t="inlineStr">
+        <is>
+          <t>Mis deudas muestra cuánto se debe actualmente, pero la experiencia se siente principalmente como una lista de obligaciones. La usuaria tiene poca visibilidad sobre cuánto ha avanzado desde que empezó y cuál es el siguiente hito dentro de su estrategia.</t>
+        </is>
+      </c>
+      <c r="E34" s="11" t="inlineStr">
+        <is>
+          <t>El módulo debe hacer visible el progreso para que pagar deudas se sienta como un proceso con avances concretos. Amy debe mostrar cuánto ha disminuido la deuda, cuál es la deuda prioritaria actual y qué hito viene después.</t>
+        </is>
+      </c>
+      <c r="F34" s="11" t="inlineStr">
+        <is>
+          <t>Como una mujer que está trabajando mes a mes para salir de deudas, quiero ver cuánto he avanzado y cuál es mi próximo objetivo, para sentir que mis pagos están produciendo progreso y mantenerme motivada.</t>
+        </is>
+      </c>
+      <c r="G34" s="11" t="inlineStr">
+        <is>
+          <t>Incorporar un resumen de progreso basado en saldos reales registrados: saldo inicial, saldo actual y reducción acumulada. Destacar la deuda prioritaria y un siguiente objetivo concreto, por ejemplo completar el pago del mes, realizar un abono adicional o liquidar la deuda prioritaria. Cuando una deuda llegue a $0, mostrar una celebración y actualizar automáticamente cuál pasa a ser la siguiente prioridad según la metodología.</t>
+        </is>
+      </c>
+      <c r="H34" s="11" t="inlineStr">
+        <is>
+          <t>Evitar mensajes que generen culpa si el progreso es lento. Celebrar constancia y cumplimiento, no únicamente grandes pagos. No mostrar fechas exactas de liquidación si no hay datos suficientes para estimarlas de manera responsable.</t>
+        </is>
+      </c>
+      <c r="I34" s="11" t="inlineStr">
+        <is>
+          <t>Aumentar motivación, retención y continuidad en el plan de deuda.</t>
+        </is>
+      </c>
+      <c r="J34" s="11" t="inlineStr">
+        <is>
+          <t>La usuaria percibe avance, entiende cuál es su siguiente meta y mantiene claridad sobre la estrategia.</t>
+        </is>
+      </c>
+      <c r="K34" s="11" t="inlineStr">
+        <is>
+          <t>El módulo muestra progreso basado en saldos reales, identifica la prioridad vigente y actualiza el siguiente objetivo al cambiar o liquidar una deuda.</t>
+        </is>
+      </c>
+      <c r="L34" s="11" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M34" s="11" t="inlineStr">
         <is>
           <t>Pendiente</t>
         </is>

</xml_diff>

<commit_message>
docs: marcar 4.13 y 4.14 como Completo en el roadmap
</commit_message>
<xml_diff>
--- a/docs/roadmap/Finance-BFF-Experience-Roadmap.xlsx
+++ b/docs/roadmap/Finance-BFF-Experience-Roadmap.xlsx
@@ -2963,7 +2963,7 @@
       </c>
       <c r="M38" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completo</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="M39" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: marcar 4.17 y 4.18 como Completo en el roadmap
</commit_message>
<xml_diff>
--- a/docs/roadmap/Finance-BFF-Experience-Roadmap.xlsx
+++ b/docs/roadmap/Finance-BFF-Experience-Roadmap.xlsx
@@ -3231,7 +3231,7 @@
       </c>
       <c r="M42" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completo</t>
         </is>
       </c>
     </row>
@@ -3298,7 +3298,7 @@
       </c>
       <c r="M43" s="9" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completo</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: flujo de caja completo — semanal, reservas guardadas y saldo explicado (roadmap 5.1-5.10)
- 5.1: ingreso semanal con fecha de inicio (migración 20260926); el motor lo proyecta cada 7 días.
- 5.5/5.6/5.9: la reserva del periodo se guarda o actualiza sola cuando hay faltante, se borra si ya no
  hace falta, y se puede marcar como apartada. Solo cuenta una reserva que existe (5.6 simplificado:
  no hay construcción progresiva sobre varios ciclos todavía).
- 5.8: el dashboard explica el saldo en cuenta y cuánto ya está apartado; calcularDisponible resta reservas.
- 5.10: ahorro y cajitas usan el mismo disponible (ya neto de reservas).
- Corrige una carrera: solo la recarga más reciente escribe la reserva, y la lista se relee después de sincronizar.
- Pruebas: tests/ciclos/run.cjs (12 checks del motor) y prueba e2e en navegador (6 checks) con verificación en base.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap/Finance-BFF-Experience-Roadmap.xlsx
+++ b/docs/roadmap/Finance-BFF-Experience-Roadmap.xlsx
@@ -24,17 +24,15 @@
     </font>
     <font>
       <name val="Arial"/>
-      <family val="2"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
-      <family val="2"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -54,6 +52,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF99CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.7999816888943144"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -130,7 +133,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -174,12 +177,88 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <colors/>
+  <colors>
+    <indexedColors>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00000000"/>
+      <rgbColor rgb="00FFFFFF"/>
+      <rgbColor rgb="00FF0000"/>
+      <rgbColor rgb="0000FF00"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008000"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00808000"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="00C0C0C0"/>
+      <rgbColor rgb="00808080"/>
+      <rgbColor rgb="009999FF"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00FFFFCC"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00660066"/>
+      <rgbColor rgb="00FF8080"/>
+      <rgbColor rgb="000066CC"/>
+      <rgbColor rgb="00CCCCFF"/>
+      <rgbColor rgb="00000080"/>
+      <rgbColor rgb="00FF00FF"/>
+      <rgbColor rgb="00FFFF00"/>
+      <rgbColor rgb="0000FFFF"/>
+      <rgbColor rgb="00800080"/>
+      <rgbColor rgb="00800000"/>
+      <rgbColor rgb="00008080"/>
+      <rgbColor rgb="000000FF"/>
+      <rgbColor rgb="0000CCFF"/>
+      <rgbColor rgb="00CCFFFF"/>
+      <rgbColor rgb="00CCFFCC"/>
+      <rgbColor rgb="00FFFF99"/>
+      <rgbColor rgb="0099CCFF"/>
+      <rgbColor rgb="00FF99CC"/>
+      <rgbColor rgb="00CC99FF"/>
+      <rgbColor rgb="00FFCC99"/>
+      <rgbColor rgb="003366FF"/>
+      <rgbColor rgb="0033CCCC"/>
+      <rgbColor rgb="0099CC00"/>
+      <rgbColor rgb="00FFCC00"/>
+      <rgbColor rgb="00FF9900"/>
+      <rgbColor rgb="00FF6600"/>
+      <rgbColor rgb="00666699"/>
+      <rgbColor rgb="00969696"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
+    </indexedColors>
+  </colors>
 </styleSheet>
 </file>
 
@@ -403,7 +482,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M45"/>
+  <dimension ref="A1:M55"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="13.8"/>
   <cols>
     <col width="24" customWidth="1" style="4" min="1" max="1"/>
@@ -421,7 +500,7 @@
     <col width="8.88671875" customWidth="1" style="4" min="16" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.2" customFormat="1" customHeight="1" s="2">
+    <row r="1" ht="17.7" customFormat="1" customHeight="1" s="2">
       <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Epic</t>
@@ -488,7 +567,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="42.45" customHeight="1">
+    <row r="2" ht="33.9" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
@@ -555,7 +634,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="35.25" customHeight="1">
+    <row r="3" ht="28.2" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
@@ -622,7 +701,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="28.2" customHeight="1">
+    <row r="4" ht="22.5" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
@@ -689,7 +768,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="35.25" customHeight="1">
+    <row r="5" ht="28.2" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
@@ -756,7 +835,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="35.25" customHeight="1">
+    <row r="6" ht="28.2" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
@@ -823,7 +902,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="28.2" customHeight="1">
+    <row r="7" ht="22.5" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
@@ -890,7 +969,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="35.25" customHeight="1">
+    <row r="8" ht="28.2" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
@@ -957,7 +1036,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="61.5" customHeight="1">
+    <row r="9" ht="49.2" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1024,7 +1103,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="61.5" customHeight="1">
+    <row r="10" ht="49.2" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1091,7 +1170,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="61.5" customHeight="1">
+    <row r="11" ht="49.2" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1158,7 +1237,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="61.5" customHeight="1">
+    <row r="12" ht="49.2" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1225,7 +1304,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="61.5" customHeight="1">
+    <row r="13" ht="49.2" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1292,7 +1371,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="61.5" customHeight="1">
+    <row r="14" ht="49.2" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Acompañamiento después del onboarding</t>
@@ -1359,7 +1438,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="61.5" customHeight="1">
+    <row r="15" ht="49.2" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Hábitos financieros y conexión con el banco</t>
@@ -1426,7 +1505,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="61.5" customHeight="1">
+    <row r="16" ht="49.2" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Hábitos financieros y conexión con el banco</t>
@@ -1493,7 +1572,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="61.5" customHeight="1">
+    <row r="17" ht="49.2" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Acompañamiento después del onboarding</t>
@@ -1560,7 +1639,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="79.5" customHeight="1">
+    <row r="18" ht="63.6" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1627,7 +1706,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="79.5" customHeight="1">
+    <row r="19" ht="63.6" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1694,7 +1773,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="79.5" customHeight="1">
+    <row r="20" ht="63.6" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1761,7 +1840,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="79.5" customHeight="1">
+    <row r="21" ht="63.6" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1828,7 +1907,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="79.5" customHeight="1">
+    <row r="22" ht="63.6" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1895,7 +1974,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="79.5" customHeight="1">
+    <row r="23" ht="63.6" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1962,7 +2041,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="79.5" customHeight="1">
+    <row r="24" ht="63.6" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -2029,7 +2108,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="79.5" customHeight="1">
+    <row r="25" ht="63.6" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -2096,7 +2175,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="79.5" customHeight="1">
+    <row r="26" ht="63.6" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Dashboard</t>
@@ -2163,7 +2242,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="79.5" customHeight="1">
+    <row r="27" ht="63.6" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Dashboard</t>
@@ -2230,7 +2309,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="79.5" customHeight="1">
+    <row r="28" ht="63.6" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
           <t>Dashboard</t>
@@ -2297,7 +2376,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="79.5" customHeight="1">
+    <row r="29" ht="63.6" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Dashboard</t>
@@ -2364,7 +2443,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="111.9" customHeight="1">
+    <row r="30" ht="89.55" customHeight="1">
       <c r="A30" s="7" t="inlineStr">
         <is>
           <t>Dashboard | Mis deudas</t>
@@ -2431,7 +2510,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="111.9" customHeight="1">
+    <row r="31" ht="89.55" customHeight="1">
       <c r="A31" s="7" t="inlineStr">
         <is>
           <t>Dashboard | Mis deudas</t>
@@ -2498,7 +2577,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="111.9" customHeight="1">
+    <row r="32" ht="89.55" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
         <is>
           <t>Dashboard | Mis deudas</t>
@@ -2565,7 +2644,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="139.95" customHeight="1">
+    <row r="33" ht="111.9" customHeight="1">
       <c r="A33" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis deudas</t>
@@ -2632,7 +2711,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="111.9" customHeight="1">
+    <row r="34" ht="89.55" customHeight="1">
       <c r="A34" s="10" t="inlineStr">
         <is>
           <t>Dashboard | Mis deudas</t>
@@ -2699,7 +2778,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="132" customHeight="1">
+    <row r="35" ht="105.6" customHeight="1">
       <c r="A35" s="12" t="inlineStr">
         <is>
           <t>Dashboard</t>
@@ -2766,7 +2845,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="132" customHeight="1">
+    <row r="36" ht="105.6" customHeight="1">
       <c r="A36" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis gastos</t>
@@ -2833,7 +2912,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="132" customHeight="1">
+    <row r="37" ht="105.6" customHeight="1">
       <c r="A37" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis cajitas</t>
@@ -2900,7 +2979,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="132" customHeight="1">
+    <row r="38" ht="105.6" customHeight="1">
       <c r="A38" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis cajitas</t>
@@ -2967,7 +3046,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="132" customHeight="1">
+    <row r="39" ht="105.6" customHeight="1">
       <c r="A39" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis ahorros</t>
@@ -3034,7 +3113,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="132" customHeight="1">
+    <row r="40" ht="105.6" customHeight="1">
       <c r="A40" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis cajitas</t>
@@ -3101,7 +3180,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="132" customHeight="1">
+    <row r="41" ht="105.6" customHeight="1">
       <c r="A41" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis ahorros</t>
@@ -3168,7 +3247,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="132" customHeight="1">
+    <row r="42" ht="105.6" customHeight="1">
       <c r="A42" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis bolsitas</t>
@@ -3235,7 +3314,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="132" customHeight="1">
+    <row r="43" ht="105.6" customHeight="1">
       <c r="A43" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis cajitas</t>
@@ -3302,7 +3381,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="132" customHeight="1">
+    <row r="44" ht="105.6" customHeight="1">
       <c r="A44" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis deudas</t>
@@ -3369,7 +3448,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="132" customHeight="1">
+    <row r="45" ht="105.6" customHeight="1">
       <c r="A45" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis deudas</t>
@@ -3431,6 +3510,676 @@
         </is>
       </c>
       <c r="M45" s="9" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="105.6" customFormat="1" customHeight="1" s="17">
+      <c r="A46" s="15" t="inlineStr">
+        <is>
+          <t>Flujo de caja y ciclos de ingreso</t>
+        </is>
+      </c>
+      <c r="B46" s="15" t="inlineStr">
+        <is>
+          <t>5.1</t>
+        </is>
+      </c>
+      <c r="C46" s="15" t="inlineStr">
+        <is>
+          <t>Identificar la frecuencia con la que la usuaria recibe sus ingresos</t>
+        </is>
+      </c>
+      <c r="D46" s="16" t="inlineStr">
+        <is>
+          <t>El onboarding conoce cuánto dinero recibe la usuaria, pero no distingue con suficiente detalle la frecuencia con la que ese dinero entra. Dos usuarias con el mismo ingreso mensual pueden vivir realidades muy diferentes si una recibe todo una vez al mes y otra recibe varios pagos durante el mes.</t>
+        </is>
+      </c>
+      <c r="E46" s="16" t="inlineStr">
+        <is>
+          <t>Durante el registro de ingresos, Amy debe entender cómo recibe el dinero la usuaria antes de construir su plan financiero. Debe reconocer frecuencias como mensual, quincenal, cada dos semanas, semanal, variable u otra frecuencia que la usuaria necesite.</t>
+        </is>
+      </c>
+      <c r="F46" s="16" t="inlineStr">
+        <is>
+          <t>Como una mujer que no recibe todo mi ingreso una sola vez al mes, quiero contarle a Amy con qué frecuencia me pagan, para que mi plan financiero refleje cómo funciona realmente mi dinero y no solo cuánto recibo en total.</t>
+        </is>
+      </c>
+      <c r="G46" s="16" t="inlineStr">
+        <is>
+          <t>Agregar la frecuencia de pago como parte de la configuración de cada fuente de ingreso. Permitir seleccionar mensual, quincenal, cada dos semanas, semanal, variable u otra. La frecuencia debe guardarse por fuente de ingreso porque una misma usuaria puede recibir ingresos con ciclos diferentes. La selección debe alimentar posteriormente la construcción de los periodos de flujo de caja.</t>
+        </is>
+      </c>
+      <c r="H46" s="16" t="inlineStr">
+        <is>
+          <t>Explicar las opciones con lenguaje cotidiano. No asumir que quincenal y cada dos semanas significan lo mismo. Si la usuaria tiene varias fuentes de ingreso, cada una debe poder tener su propia frecuencia.</t>
+        </is>
+      </c>
+      <c r="I46" s="16" t="inlineStr">
+        <is>
+          <t>Construir planes financieros que representen el momento real en el que el dinero entra y mejorar la precisión de las recomendaciones de Amy.</t>
+        </is>
+      </c>
+      <c r="J46" s="16" t="inlineStr">
+        <is>
+          <t>Amy conoce no solo cuánto gana la usuaria sino también el ritmo con el que recibe cada ingreso.</t>
+        </is>
+      </c>
+      <c r="K46" s="16" t="inlineStr">
+        <is>
+          <t>Cada fuente de ingreso conserva su frecuencia y Amy utiliza esa información para construir los periodos de disponibilidad de dinero.</t>
+        </is>
+      </c>
+      <c r="L46" s="16" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M46" s="16" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="105.6" customFormat="1" customHeight="1" s="17">
+      <c r="A47" s="15" t="inlineStr">
+        <is>
+          <t>Flujo de caja y ciclos de ingreso</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>5.2</t>
+        </is>
+      </c>
+      <c r="C47" s="15" t="inlineStr">
+        <is>
+          <t>Registrar el monto y la fecha aproximada de cada pago</t>
+        </is>
+      </c>
+      <c r="D47" s="16" t="inlineStr">
+        <is>
+          <t>Conocer que un ingreso es quincenal no permite saber cuánto recibe la usuaria en cada pago ni cuándo lo recibe. El sistema podría asumir incorrectamente una distribución igual aunque en la vida real un pago represente, por ejemplo, 40 por ciento del ingreso y el otro 60 por ciento.</t>
+        </is>
+      </c>
+      <c r="E47" s="16" t="inlineStr">
+        <is>
+          <t>Amy debe permitir registrar cuánto dinero llega en cada pago y en qué fecha o momento aproximado del mes suele llegar, sin asumir que los pagos tienen el mismo valor.</t>
+        </is>
+      </c>
+      <c r="F47" s="16" t="inlineStr">
+        <is>
+          <t>Como una mujer que recibe diferentes montos durante el mes, quiero indicar cuánto recibo en cada pago y cuándo suele llegar, para que Amy pueda organizar mis obligaciones con el dinero que realmente tendré disponible en cada momento.</t>
+        </is>
+      </c>
+      <c r="G47" s="16" t="inlineStr">
+        <is>
+          <t>Cuando una fuente tenga más de un pago por mes, solicitar monto y fecha aproximada de cada pago. No dividir automáticamente el ingreso mensual en partes iguales. Permitir editar estos datos cuando cambie el empleo, el salario o la estructura de pagos. Para ingresos variables, permitir registrar una estimación y actualizar el monto real cuando se reciba.</t>
+        </is>
+      </c>
+      <c r="H47" s="16" t="inlineStr">
+        <is>
+          <t>Mantener el flujo simple y progresivo. Mostrar el total mensual resultante para que la usuaria pueda validar que la información registrada tiene sentido. Evitar exigir fechas exactas cuando la usuaria solo conoce un rango aproximado.</t>
+        </is>
+      </c>
+      <c r="I47" s="16" t="inlineStr">
+        <is>
+          <t>Dar a Amy información temporal suficiente para organizar el dinero de forma realista.</t>
+        </is>
+      </c>
+      <c r="J47" s="16" t="inlineStr">
+        <is>
+          <t>El plan refleja la distribución real de los ingresos dentro del mes, incluso cuando los pagos no son iguales.</t>
+        </is>
+      </c>
+      <c r="K47" s="16" t="inlineStr">
+        <is>
+          <t>Los pagos pueden tener montos diferentes, conservan su fecha aproximada y el total mensual se calcula correctamente a partir de ellos.</t>
+        </is>
+      </c>
+      <c r="L47" s="16" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M47" s="16" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="105.6" customFormat="1" customHeight="1" s="17">
+      <c r="A48" s="15" t="inlineStr">
+        <is>
+          <t>Flujo de caja y ciclos de ingreso</t>
+        </is>
+      </c>
+      <c r="B48" s="15" t="inlineStr">
+        <is>
+          <t>5.3</t>
+        </is>
+      </c>
+      <c r="C48" s="15" t="inlineStr">
+        <is>
+          <t>Registrar cuándo deben pagarse las obligaciones recurrentes</t>
+        </is>
+      </c>
+      <c r="D48" s="16" t="inlineStr">
+        <is>
+          <t>Los gastos fijos indican cuánto debe pagar la usuaria, pero el monto mensual por sí solo no permite saber qué ingreso debe cubrir cada obligación. Esto puede ocultar periodos en los que la usuaria se queda con muy poco dinero aunque el mes completo cierre positivamente.</t>
+        </is>
+      </c>
+      <c r="E48" s="16" t="inlineStr">
+        <is>
+          <t>Amy debe conocer aproximadamente cuándo vence o se paga cada obligación recurrente para relacionarla con los ingresos disponibles antes de esa fecha.</t>
+        </is>
+      </c>
+      <c r="F48" s="16" t="inlineStr">
+        <is>
+          <t>Como una mujer que tiene varias obligaciones en momentos diferentes del mes, quiero indicarle a Amy cuándo debo pagarlas, para que me ayude a preparar el dinero antes de cada vencimiento.</t>
+        </is>
+      </c>
+      <c r="G48" s="16" t="inlineStr">
+        <is>
+          <t>Agregar fecha de pago o vencimiento a los gastos fijos y demás obligaciones recurrentes que afecten el flujo de caja. Permitir una fecha exacta o un momento aproximado del mes cuando corresponda. Usar esta información para asignar cada obligación al periodo de ingreso que debe financiarla. Permitir modificar la fecha cuando cambien las condiciones del servicio o contrato.</t>
+        </is>
+      </c>
+      <c r="H48" s="16" t="inlineStr">
+        <is>
+          <t>No convertir el onboarding en una captura interminable de fechas. Pedir este dato únicamente donde sea útil para el flujo de caja y permitir completarlo después si la usuaria no lo conoce en ese momento.</t>
+        </is>
+      </c>
+      <c r="I48" s="16" t="inlineStr">
+        <is>
+          <t>Permitir que Amy anticipe necesidades de efectivo y reduzca desbalances dentro del mes.</t>
+        </is>
+      </c>
+      <c r="J48" s="16" t="inlineStr">
+        <is>
+          <t>La usuaria puede ver sus obligaciones en relación con los ingresos que estarán disponibles antes de pagarlas.</t>
+        </is>
+      </c>
+      <c r="K48" s="16" t="inlineStr">
+        <is>
+          <t>Las obligaciones recurrentes conservan una fecha o periodo de pago y Amy puede asociarlas correctamente con los ciclos de ingreso.</t>
+        </is>
+      </c>
+      <c r="L48" s="16" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M48" s="16" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="105.6" customFormat="1" customHeight="1" s="17">
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>Flujo de caja y ciclos de ingreso</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="inlineStr">
+        <is>
+          <t>5.4</t>
+        </is>
+      </c>
+      <c r="C49" s="15" t="inlineStr">
+        <is>
+          <t>Detectar falta de liquidez entre un ingreso y el siguiente</t>
+        </is>
+      </c>
+      <c r="D49" s="16" t="inlineStr">
+        <is>
+          <t>Una usuaria puede tener capacidad financiera positiva al finalizar el mes y aun así quedarse prácticamente sin dinero durante varios días porque sus obligaciones se concentran antes de uno de sus pagos. El cálculo mensual puede mostrar dinero disponible y ocultar este problema.</t>
+        </is>
+      </c>
+      <c r="E49" s="16" t="inlineStr">
+        <is>
+          <t>Antes de recomendar ahorro o mostrar dinero libre, Amy debe revisar cada periodo entre ingresos y detectar si la usuaria tendrá suficiente dinero para cubrir obligaciones y gastos necesarios hasta recibir el siguiente pago.</t>
+        </is>
+      </c>
+      <c r="F49" s="16" t="inlineStr">
+        <is>
+          <t>Como una mujer cuyos ingresos mensuales sí alcanzan pero están distribuidos de forma desigual, quiero que Amy detecte cuando una parte del mes queda demasiado ajustada, para no creer que tengo dinero disponible cuando todavía necesito cubrir los días antes de mi próximo pago.</t>
+        </is>
+      </c>
+      <c r="G49" s="16" t="inlineStr">
+        <is>
+          <t>Construir periodos de flujo de caja desde cada ingreso hasta el siguiente. Para cada periodo calcular dinero inicial, ingresos recibidos, obligaciones que vencen durante ese intervalo, reservas ya asignadas y monto restante para los gastos necesarios del periodo. Si el resultado deja a la usuaria sin liquidez suficiente, identificar el desbalance antes de calcular capacidad de ahorro. No clasificar automáticamente el caso como falta de ingresos mensuales si el problema es temporal.</t>
+        </is>
+      </c>
+      <c r="H49" s="16" t="inlineStr">
+        <is>
+          <t>Comunicar el hallazgo sin alarmar ni culpabilizar. Explicar la diferencia entre que el mes alcance y que el dinero esté disponible en el momento correcto. Evitar mostrar como libre dinero que ya se necesita para un periodo futuro.</t>
+        </is>
+      </c>
+      <c r="I49" s="16" t="inlineStr">
+        <is>
+          <t>Evitar recomendaciones de ahorro que comprometan la capacidad de la usuaria para llegar a su siguiente ingreso.</t>
+        </is>
+      </c>
+      <c r="J49" s="16" t="inlineStr">
+        <is>
+          <t>Amy distingue entre capacidad mensual y liquidez dentro del mes y puede intervenir antes de que aparezca un periodo sin dinero.</t>
+        </is>
+      </c>
+      <c r="K49" s="16" t="inlineStr">
+        <is>
+          <t>El sistema identifica periodos con insuficiente liquidez aunque el balance mensual sea positivo y no recomienda como disponible el dinero necesario para cubrirlos.</t>
+        </is>
+      </c>
+      <c r="L49" s="16" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M49" s="16" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="105.6" customFormat="1" customHeight="1" s="17">
+      <c r="A50" s="15" t="inlineStr">
+        <is>
+          <t>Flujo de caja y ciclos de ingreso</t>
+        </is>
+      </c>
+      <c r="B50" s="15" t="inlineStr">
+        <is>
+          <t>5.5</t>
+        </is>
+      </c>
+      <c r="C50" s="15" t="inlineStr">
+        <is>
+          <t>Crear una reserva para equilibrar el siguiente periodo de ingreso</t>
+        </is>
+      </c>
+      <c r="D50" s="16" t="inlineStr">
+        <is>
+          <t>Cuando un periodo del mes queda muy ajustado y otro tiene mayor holgura, la usuaria puede necesitar conservar parte del ingreso más fuerte para utilizarlo después. Sin esta reserva, el excedente puede parecer disponible para ahorro o gasto aunque tenga un propósito próximo.</t>
+        </is>
+      </c>
+      <c r="E50" s="16" t="inlineStr">
+        <is>
+          <t>Si Amy detecta un desbalance entre periodos, debe calcular cuánto dinero conviene reservar desde el periodo más holgado para complementar el siguiente y permitir que la usuaria llegue a su próximo ingreso con el dinero necesario.</t>
+        </is>
+      </c>
+      <c r="F50" s="16" t="inlineStr">
+        <is>
+          <t>Como una mujer que recibe más dinero en una parte del mes que en otra, quiero que Amy me diga cuánto debo dejar preparado para mi siguiente periodo, para no quedarme sin liquidez aunque mi presupuesto mensual sí alcance.</t>
+        </is>
+      </c>
+      <c r="G50" s="16" t="inlineStr">
+        <is>
+          <t>Calcular una reserva de transición entre periodos cuando sea necesaria. La reserva debe considerar las obligaciones y necesidades que ocurren antes del siguiente ingreso suficiente. Mostrar cuánto debe apartarse, desde qué ingreso debe reservarse y para qué periodo se está protegiendo. Restar esta reserva del dinero realmente disponible antes de calcular nuevas bolsitas o ahorro adicional. Recalcularla cuando cambien ingresos, fechas u obligaciones.</t>
+        </is>
+      </c>
+      <c r="H50" s="16" t="inlineStr">
+        <is>
+          <t>No presentar esta reserva como ahorro porque su propósito es financiar gastos próximos. Debe sentirse como dinero con destino. Explicar claramente que la usuaria no está perdiendo capacidad financiera, sino moviendo dinero en el tiempo para que esté disponible cuando lo necesite.</t>
+        </is>
+      </c>
+      <c r="I50" s="16" t="inlineStr">
+        <is>
+          <t>Reducir la dependencia de crédito para cubrir desbalances temporales y ayudar a la usuaria a anticiparse a sus necesidades.</t>
+        </is>
+      </c>
+      <c r="J50" s="16" t="inlineStr">
+        <is>
+          <t>La usuaria llega al siguiente periodo con dinero previamente preparado y entiende por qué ese monto no está disponible para otros objetivos.</t>
+        </is>
+      </c>
+      <c r="K50" s="16" t="inlineStr">
+        <is>
+          <t>La reserva se calcula cuando existe un desbalance, se descuenta del dinero disponible y se actualiza cuando cambian las condiciones del flujo.</t>
+        </is>
+      </c>
+      <c r="L50" s="16" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M50" s="16" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="105.6" customFormat="1" customHeight="1" s="17">
+      <c r="A51" s="15" t="inlineStr">
+        <is>
+          <t>Flujo de caja y ciclos de ingreso</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="C51" s="15" t="inlineStr">
+        <is>
+          <t>Acompañar el primer ciclo cuando todavía no existe una reserva previa</t>
+        </is>
+      </c>
+      <c r="D51" s="16" t="inlineStr">
+        <is>
+          <t>Una usuaria que acaba de cambiar de trabajo o de frecuencia de pago puede necesitar una reserva entre periodos, pero durante su primer ciclo todavía no ha tenido un ingreso anterior desde el cual construirla. El sistema no debe comportarse como si esa reserva ya existiera.</t>
+        </is>
+      </c>
+      <c r="E51" s="16" t="inlineStr">
+        <is>
+          <t>Amy debe reconocer el primer ciclo como una etapa de transición y mostrar con claridad cuánto falta para estabilizar el flujo, qué puede cubrir con el dinero actual y cómo construir progresivamente la reserva necesaria.</t>
+        </is>
+      </c>
+      <c r="F51" s="16" t="inlineStr">
+        <is>
+          <t>Como una mujer que acaba de empezar a recibir mi salario con una nueva frecuencia, quiero que Amy reconozca que todavía no tengo dinero preparado del periodo anterior, para recibir un plan realista mientras organizo mi nuevo ciclo.</t>
+        </is>
+      </c>
+      <c r="G51" s="16" t="inlineStr">
+        <is>
+          <t>Detectar cuando la usuaria está iniciando un nuevo esquema de ingresos y no cuenta con la reserva calculada. Crear un plan de transición que muestre la necesidad temporal y permita construir la reserva en uno o varios ingresos posteriores según la capacidad disponible. No asumir el uso de tarjeta de crédito ni recomendar endeudamiento como solución predeterminada. Una vez completada la reserva, cambiar automáticamente al funcionamiento regular.</t>
+        </is>
+      </c>
+      <c r="H51" s="16" t="inlineStr">
+        <is>
+          <t>Evitar hacer sentir a la usuaria que su plan está mal por una situación temporal. Diferenciar claramente transición de funcionamiento habitual y mostrar progreso hacia la estabilización.</t>
+        </is>
+      </c>
+      <c r="I51" s="16" t="inlineStr">
+        <is>
+          <t>Acompañar cambios laborales o de frecuencia de pago sin generar recomendaciones inviables durante el primer ciclo.</t>
+        </is>
+      </c>
+      <c r="J51" s="16" t="inlineStr">
+        <is>
+          <t>La usuaria entiende por qué el primer periodo es diferente y cómo llegará a una estructura estable sin que Amy presuponga dinero que todavía no existe.</t>
+        </is>
+      </c>
+      <c r="K51" s="16" t="inlineStr">
+        <is>
+          <t>El sistema identifica el primer ciclo, no contabiliza una reserva inexistente y permite construirla progresivamente hasta activar el flujo regular.</t>
+        </is>
+      </c>
+      <c r="L51" s="16" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M51" s="16" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="105.6" customFormat="1" customHeight="1" s="17">
+      <c r="A52" s="15" t="inlineStr">
+        <is>
+          <t>Flujo de caja y ciclos de ingreso</t>
+        </is>
+      </c>
+      <c r="B52" s="15" t="inlineStr">
+        <is>
+          <t>5.7</t>
+        </is>
+      </c>
+      <c r="C52" s="15" t="inlineStr">
+        <is>
+          <t>Mostrar en el dashboard el plan hasta el próximo ingreso</t>
+        </is>
+      </c>
+      <c r="D52" s="16" t="inlineStr">
+        <is>
+          <t>El dashboard se organiza principalmente alrededor del mes, pero una usuaria que recibe varios pagos necesita saber qué debe hacer con el dinero disponible ahora y qué debe cubrir antes de recibir el siguiente ingreso.</t>
+        </is>
+      </c>
+      <c r="E52" s="16" t="inlineStr">
+        <is>
+          <t>Además de conservar la visión mensual, el dashboard debe mostrar un plan sencillo para el periodo actual con el próximo ingreso, las obligaciones que deben cubrirse antes de esa fecha, el dinero reservado y el monto que realmente puede utilizarse.</t>
+        </is>
+      </c>
+      <c r="F52" s="16" t="inlineStr">
+        <is>
+          <t>Como una mujer que recibe varios pagos durante el mes, quiero ver qué debo cubrir hasta mi próximo ingreso, para tomar decisiones con el dinero que tengo hoy sin perder de vista mi plan mensual.</t>
+        </is>
+      </c>
+      <c r="G52" s="16" t="inlineStr">
+        <is>
+          <t>Crear un bloque de periodo actual dentro del dashboard para usuarias cuya frecuencia de ingreso lo requiera. Mostrar fecha aproximada del próximo ingreso, obligaciones pendientes antes de esa fecha, reservas asignadas y dinero disponible para ese periodo. Al llegar un nuevo ingreso, avanzar al siguiente periodo y recalcular la información. Mantener la visión mensual como contexto general.</t>
+        </is>
+      </c>
+      <c r="H52" s="16" t="inlineStr">
+        <is>
+          <t>Evitar duplicar todo el dashboard. La vista del periodo debe responder una pregunta concreta: qué necesito hacer con mi dinero hasta que vuelva a recibir ingresos. Mantener jerarquía visual clara entre mes y periodo actual.</t>
+        </is>
+      </c>
+      <c r="I52" s="16" t="inlineStr">
+        <is>
+          <t>Convertir el dashboard en una herramienta útil para decisiones cotidianas y aumentar la frecuencia de uso de Amy.</t>
+        </is>
+      </c>
+      <c r="J52" s="16" t="inlineStr">
+        <is>
+          <t>La usuaria entiende su mes completo y al mismo tiempo sabe qué debe hacer con el dinero disponible hasta el próximo pago.</t>
+        </is>
+      </c>
+      <c r="K52" s="16" t="inlineStr">
+        <is>
+          <t>El dashboard muestra el periodo vigente, el siguiente ingreso y las obligaciones que deben cubrirse antes de recibirlo con datos consistentes con el plan mensual.</t>
+        </is>
+      </c>
+      <c r="L52" s="16" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M52" s="16" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="105.6" customFormat="1" customHeight="1" s="17">
+      <c r="A53" s="15" t="inlineStr">
+        <is>
+          <t>Flujo de caja y ciclos de ingreso</t>
+        </is>
+      </c>
+      <c r="B53" s="15" t="inlineStr">
+        <is>
+          <t>5.8</t>
+        </is>
+      </c>
+      <c r="C53" s="15" t="inlineStr">
+        <is>
+          <t>Diferenciar saldo en cuenta de dinero realmente disponible</t>
+        </is>
+      </c>
+      <c r="D53" s="16" t="inlineStr">
+        <is>
+          <t>Una usuaria puede ver un saldo alto en su cuenta después de recibir un pago, pero una parte de ese dinero puede estar destinada a obligaciones o a complementar el siguiente periodo. Mostrar todo el saldo como disponible puede llevarla a gastar o ahorrar dinero que ya tiene un propósito.</t>
+        </is>
+      </c>
+      <c r="E53" s="16" t="inlineStr">
+        <is>
+          <t>Amy debe separar conceptualmente el dinero que existe en la cuenta del dinero que realmente está libre para decisiones nuevas después de proteger obligaciones y reservas.</t>
+        </is>
+      </c>
+      <c r="F53" s="16" t="inlineStr">
+        <is>
+          <t>Como una mujer que acaba de recibir mi salario, quiero saber cuánto de ese dinero realmente puedo usar, para no confundir tener dinero en la cuenta con tener dinero libre.</t>
+        </is>
+      </c>
+      <c r="G53" s="16" t="inlineStr">
+        <is>
+          <t>Actualizar la lógica de Dinero disponible para excluir obligaciones pendientes, cajitas, compromisos confirmados y reservas necesarias para periodos futuros según las reglas vigentes del producto. Cuando exista dinero reservado para el siguiente periodo, mostrarlo de forma separada y explicar su propósito. Todos los módulos que utilicen Dinero disponible deben consumir la misma lógica central.</t>
+        </is>
+      </c>
+      <c r="H53" s="16" t="inlineStr">
+        <is>
+          <t>Usar términos muy claros y consistentes. La usuaria debe poder entender por qué su saldo bancario puede ser mayor que el monto que Amy considera disponible sin sentir que el dinero desapareció.</t>
+        </is>
+      </c>
+      <c r="I53" s="16" t="inlineStr">
+        <is>
+          <t>Evitar decisiones basadas en una falsa sensación de liquidez y fortalecer la confianza en los cálculos de Amy.</t>
+        </is>
+      </c>
+      <c r="J53" s="16" t="inlineStr">
+        <is>
+          <t>La usuaria sabe qué parte de su dinero tiene destino y qué parte puede utilizar para nuevas decisiones.</t>
+        </is>
+      </c>
+      <c r="K53" s="16" t="inlineStr">
+        <is>
+          <t>Dinero disponible excluye correctamente las reservas y obligaciones comprometidas y la diferencia puede explicarse desde el dashboard.</t>
+        </is>
+      </c>
+      <c r="L53" s="16" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M53" s="16" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="105.6" customFormat="1" customHeight="1" s="17">
+      <c r="A54" s="15" t="inlineStr">
+        <is>
+          <t>Flujo de caja y ciclos de ingreso</t>
+        </is>
+      </c>
+      <c r="B54" s="15" t="inlineStr">
+        <is>
+          <t>5.9</t>
+        </is>
+      </c>
+      <c r="C54" s="15" t="inlineStr">
+        <is>
+          <t>Confirmar que la reserva del siguiente periodo ya fue apartada</t>
+        </is>
+      </c>
+      <c r="D54" s="16" t="inlineStr">
+        <is>
+          <t>Amy puede calcular que una parte del ingreso debe reservarse para el siguiente periodo, pero el cálculo por sí solo no garantiza que la usuaria haya separado ese dinero en la vida real.</t>
+        </is>
+      </c>
+      <c r="E54" s="16" t="inlineStr">
+        <is>
+          <t>La usuaria debe recibir una acción concreta para apartar la reserva y poder confirmar cuando ya lo hizo, siguiendo la misma filosofía de conexión entre Amy y las acciones reales que existe en Cajitas, Bolsitas y Deudas.</t>
+        </is>
+      </c>
+      <c r="F54" s="16" t="inlineStr">
+        <is>
+          <t>Como una mujer que necesita guardar parte de este ingreso para mi siguiente periodo, quiero marcar cuando ya aparté ese dinero, para que Amy me ayude a convertir el plan en una acción real y pueda seguir mi progreso.</t>
+        </is>
+      </c>
+      <c r="G54" s="16" t="inlineStr">
+        <is>
+          <t>Cuando exista una reserva entre periodos, mostrar el monto y una instrucción para separarlo en el banco, cuenta o método que utilice la usuaria. Incluir una confirmación explícita cuando la acción esté realizada. Conservar el estado durante el periodo correspondiente y crear una nueva tarea únicamente cuando exista una nueva reserva por separar. No confundir esta acción con ahorro de largo plazo.</t>
+        </is>
+      </c>
+      <c r="H54" s="16" t="inlineStr">
+        <is>
+          <t>El texto debe ser literal y orientado a la acción. Mostrar qué cantidad debe apartarse y para qué periodo se está guardando. La confirmación debe sentirse como cumplimiento de una tarea, no como una operación bancaria automática.</t>
+        </is>
+      </c>
+      <c r="I54" s="16" t="inlineStr">
+        <is>
+          <t>Convertir la recomendación de flujo de caja en un hábito concreto y medible.</t>
+        </is>
+      </c>
+      <c r="J54" s="16" t="inlineStr">
+        <is>
+          <t>La usuaria efectivamente separa el dinero que Amy identificó como necesario para el siguiente periodo.</t>
+        </is>
+      </c>
+      <c r="K54" s="16" t="inlineStr">
+        <is>
+          <t>Cada reserva necesaria genera una acción clara, puede marcarse como realizada y conserva correctamente su estado durante el ciclo correspondiente.</t>
+        </is>
+      </c>
+      <c r="L54" s="16" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M54" s="16" t="inlineStr">
+        <is>
+          <t>Completo</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="105.6" customFormat="1" customHeight="1" s="17">
+      <c r="A55" s="15" t="inlineStr">
+        <is>
+          <t>Flujo de caja y ciclos de ingreso</t>
+        </is>
+      </c>
+      <c r="B55" s="15" t="inlineStr">
+        <is>
+          <t>5.10</t>
+        </is>
+      </c>
+      <c r="C55" s="15" t="inlineStr">
+        <is>
+          <t>Calcular el ahorro disponible después de proteger la liquidez</t>
+        </is>
+      </c>
+      <c r="D55" s="16" t="inlineStr">
+        <is>
+          <t>El excedente mensual puede parecer disponible para ahorro aunque una parte sea necesaria para complementar un periodo del mes que queda corto. Si Amy recomienda bolsitas antes de proteger esa liquidez, puede crear un plan que funciona en el total mensual pero falla durante el mes.</t>
+        </is>
+      </c>
+      <c r="E55" s="16" t="inlineStr">
+        <is>
+          <t>Amy debe determinar la capacidad de ahorro únicamente después de cubrir obligaciones y proteger el dinero necesario para llegar de forma sostenible al siguiente ingreso.</t>
+        </is>
+      </c>
+      <c r="F55" s="16" t="inlineStr">
+        <is>
+          <t>Como una mujer que quiere ahorrar sin quedarme corta antes de mi próximo pago, quiero que Amy calcule mi capacidad de ahorro después de reservar lo que necesito para vivir y cumplir mis obligaciones entre ingresos.</t>
+        </is>
+      </c>
+      <c r="G55" s="16" t="inlineStr">
+        <is>
+          <t>Incorporar las reservas de flujo de caja dentro del cálculo central de capacidad de ahorro. El orden lógico debe proteger primero las obligaciones y necesidades del periodo, después las reservas necesarias para periodos futuros y solo entonces determinar cuánto dinero puede destinarse a nuevas bolsitas u otros objetivos de ahorro. Recalcular automáticamente cuando cambien ingresos, pagos, fechas, gastos u obligaciones.</t>
+        </is>
+      </c>
+      <c r="H55" s="16" t="inlineStr">
+        <is>
+          <t>No presentar una capacidad de ahorro mayor simplemente porque existe un excedente al final del mes. Si una reserva reduce temporalmente lo disponible para ahorrar, explicar que ese dinero está protegiendo el flujo y no representa una pérdida.</t>
+        </is>
+      </c>
+      <c r="I55" s="16" t="inlineStr">
+        <is>
+          <t>Evitar planes de ahorro que obliguen a la usuaria a recurrir a deuda o quedarse sin liquidez durante el mes.</t>
+        </is>
+      </c>
+      <c r="J55" s="16" t="inlineStr">
+        <is>
+          <t>La recomendación de ahorro de Amy es sostenible tanto a nivel mensual como entre cada ingreso.</t>
+        </is>
+      </c>
+      <c r="K55" s="16" t="inlineStr">
+        <is>
+          <t>Las recomendaciones de ahorro se calculan después de las reservas necesarias y nunca utilizan dinero que Amy ya identificó como necesario antes del siguiente ingreso.</t>
+        </is>
+      </c>
+      <c r="L55" s="16" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M55" s="16" t="inlineStr">
         <is>
           <t>Completo</t>
         </is>

</xml_diff>

<commit_message>
docs: sincronizar el roadmap con el Excel del 5 de octubre
Reemplaza docs/roadmap/Finance-BFF-Experience-Roadmap.xlsx por la copia de
Descargas (61 historias, agrega 5.11-5.17 nuevas). Marca Completo lo que ya
estaba implementado y probado pero el Excel nunca reflejó: 3.2, 3.6-3.9, 4.8,
4.10-4.20.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap/Finance-BFF-Experience-Roadmap.xlsx
+++ b/docs/roadmap/Finance-BFF-Experience-Roadmap.xlsx
@@ -8,7 +8,9 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Finance BFF Experience Roadmap" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Finance BFF Experience Roadmap'!$A$1:$O$1</definedName>
+  </definedNames>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -32,7 +34,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -56,8 +58,18 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.7999816888943144"/>
-        <bgColor indexed="64"/>
+        <fgColor theme="7" tint="0.7999511703848384"/>
+        <bgColor indexed="65"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -133,7 +145,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -185,6 +197,24 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -482,7 +512,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M55"/>
+  <dimension ref="A1:M62"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="13.8"/>
   <cols>
     <col width="24" customWidth="1" style="4" min="1" max="1"/>
@@ -500,7 +530,7 @@
     <col width="8.88671875" customWidth="1" style="4" min="16" max="16384"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.7" customFormat="1" customHeight="1" s="2">
+    <row r="1" ht="14.1" customFormat="1" customHeight="1" s="2">
       <c r="A1" s="14" t="inlineStr">
         <is>
           <t>Epic</t>
@@ -567,7 +597,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="33.9" customHeight="1">
+    <row r="2" ht="27.15" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
@@ -634,7 +664,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="28.2" customHeight="1">
+    <row r="3" ht="22.5" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
@@ -701,7 +731,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="22.5" customHeight="1">
+    <row r="4" ht="18" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
@@ -768,7 +798,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="28.2" customHeight="1">
+    <row r="5" ht="22.5" customHeight="1">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
@@ -835,7 +865,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="28.2" customHeight="1">
+    <row r="6" ht="22.5" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
@@ -902,7 +932,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="22.5" customHeight="1">
+    <row r="7" ht="18" customHeight="1">
       <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
@@ -969,7 +999,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="28.2" customHeight="1">
+    <row r="8" ht="22.5" customHeight="1">
       <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Primera impresión de la Landing</t>
@@ -1036,7 +1066,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="49.2" customHeight="1">
+    <row r="9" ht="39.3" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1103,74 +1133,74 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="49.2" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
+    <row r="10" ht="39.3" customHeight="1">
+      <c r="A10" s="20" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>3.2</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>Formato inteligente para valores de dinero</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="inlineStr">
-        <is>
-          <t>Los campos monetarios no mantienen una presentación consistente mientras la usuaria escribe y algunos inputs muestran controles nativos con flechas para aumentar o disminuir números.</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr">
-        <is>
-          <t>Todos los valores de dinero deben ser fáciles de leer desde el momento en que se ingresan, mostrando el signo $ y separadores de miles de forma automática, sin controles numéricos que generen ruido visual.</t>
-        </is>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>Como una mujer que está ingresando varios valores de ingresos, gastos, cajitas y ahorros, quiero ver los montos en un formato claro mientras los escribo, para evitar errores y entender rápidamente las cantidades que estoy registrando.</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Aplicar formato monetario en todos los campos de dinero del producto: signo $ y puntos como separadores de miles. El formato debe actualizarse mientras se escribe. Eliminar las flechas nativas de incremento y decremento de los inputs numéricos y mantener el campo abierto para escritura directa.</t>
-        </is>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>El formato debe ayudar a leer, no dificultar la edición. Mantener consistencia en onboarding, dashboard y módulos posteriores.</t>
-        </is>
-      </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>Reducir errores de digitación y mejorar la comprensión de la información financiera.</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>La usuaria interpreta los montos de inmediato y encuentra una experiencia consistente en toda la plataforma.</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>Todos los campos monetarios aplicables muestran $ y separadores de miles y ninguno presenta controles nativos de incremento/decremento.</t>
-        </is>
-      </c>
-      <c r="L10" s="3" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="M10" s="3" t="inlineStr">
+      <c r="C10" s="20" t="inlineStr">
+        <is>
+          <t>Aplicar formato inteligente a todos los valores de dinero</t>
+        </is>
+      </c>
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>Finance BFF utiliza campos monetarios en diferentes módulos. Aunque el formato inteligente se identificó inicialmente durante el onboarding, en nuevas secciones todavía aparecen valores como 2000000 mientras la usuaria escribe. Esto dificulta la lectura y genera inconsistencias entre pantallas.</t>
+        </is>
+      </c>
+      <c r="E10" s="20" t="inlineStr">
+        <is>
+          <t>Todos los campos donde la usuaria ingrese o edite dinero deben aplicar el mismo formato monetario en tiempo real. La cifra debe ser fácil de leer mientras se escribe y respetar la moneda configurada por la usuaria.</t>
+        </is>
+      </c>
+      <c r="F10" s="20" t="inlineStr">
+        <is>
+          <t>Como una mujer que registra valores de dinero en diferentes partes de Finance BFF, quiero que las cifras se formateen automáticamente mientras escribo, para poder leerlas y validar fácilmente sin contar ceros.</t>
+        </is>
+      </c>
+      <c r="G10" s="20" t="inlineStr">
+        <is>
+          <t>Convertir esta regla en un estándar global del producto. Todo input monetario debe mostrar símbolo de moneda cuando corresponda y separadores de miles mientras la usuaria escribe. Para COP, por ejemplo, 2000000 debe visualizarse como $2.000.000. El valor almacenado debe mantenerse numérico para cálculos. Aplicar la regla en onboarding, ingresos, gastos, cajitas, bolsitas, deudas, plan de ingresos y cualquier nuevo módulo con montos. Evitar inputs numéricos con controles de incremento y decremento del navegador.</t>
+        </is>
+      </c>
+      <c r="H10" s="20" t="inlineStr">
+        <is>
+          <t>El formato debe ocurrir mientras la usuaria escribe y no únicamente después de guardar. Respetar la moneda seleccionada y sus convenciones. No permitir que el formateo mueva el cursor de forma confusa ni dificulte corregir una cifra.</t>
+        </is>
+      </c>
+      <c r="I10" s="20" t="inlineStr">
+        <is>
+          <t>Crear consistencia transversal, reducir errores de captura y facilitar la lectura de valores financieros.</t>
+        </is>
+      </c>
+      <c r="J10" s="20" t="inlineStr">
+        <is>
+          <t>La usuaria reconoce y valida los montos fácilmente en cualquier pantalla de Finance BFF.</t>
+        </is>
+      </c>
+      <c r="K10" s="20" t="inlineStr">
+        <is>
+          <t>Todos los campos monetarios del producto aplican el formato correspondiente durante la escritura y mantienen valores numéricos correctos para los cálculos.</t>
+        </is>
+      </c>
+      <c r="L10" s="20" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M10" s="20" t="inlineStr">
         <is>
           <t>Completo</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="49.2" customHeight="1">
+    <row r="11" ht="39.3" customHeight="1">
       <c r="A11" s="3" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1237,7 +1267,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="49.2" customHeight="1">
+    <row r="12" ht="39.3" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1304,7 +1334,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="49.2" customHeight="1">
+    <row r="13" ht="39.3" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1371,7 +1401,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="49.2" customHeight="1">
+    <row r="14" ht="39.3" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Acompañamiento después del onboarding</t>
@@ -1438,7 +1468,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="49.2" customHeight="1">
+    <row r="15" ht="39.3" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Hábitos financieros y conexión con el banco</t>
@@ -1505,7 +1535,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="49.2" customHeight="1">
+    <row r="16" ht="39.3" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Hábitos financieros y conexión con el banco</t>
@@ -1572,7 +1602,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="49.2" customHeight="1">
+    <row r="17" ht="39.3" customHeight="1">
       <c r="A17" s="3" t="inlineStr">
         <is>
           <t>Acompañamiento después del onboarding</t>
@@ -1639,7 +1669,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="63.6" customHeight="1">
+    <row r="18" ht="50.85" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1706,7 +1736,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="63.6" customHeight="1">
+    <row r="19" ht="50.85" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1773,7 +1803,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="63.6" customHeight="1">
+    <row r="20" ht="50.85" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1840,7 +1870,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="63.6" customHeight="1">
+    <row r="21" ht="50.85" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1907,7 +1937,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="63.6" customHeight="1">
+    <row r="22" ht="50.85" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -1974,7 +2004,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="63.6" customHeight="1">
+    <row r="23" ht="50.85" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -2041,7 +2071,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="63.6" customHeight="1">
+    <row r="24" ht="50.85" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -2108,7 +2138,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="63.6" customHeight="1">
+    <row r="25" ht="50.85" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>Onboarding Happy Path</t>
@@ -2175,7 +2205,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="63.6" customHeight="1">
+    <row r="26" ht="50.85" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
         <is>
           <t>Dashboard</t>
@@ -2242,7 +2272,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="63.6" customHeight="1">
+    <row r="27" ht="50.85" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
           <t>Dashboard</t>
@@ -2309,7 +2339,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="63.6" customHeight="1">
+    <row r="28" ht="50.85" customHeight="1">
       <c r="A28" s="5" t="inlineStr">
         <is>
           <t>Dashboard</t>
@@ -2376,7 +2406,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="63.6" customHeight="1">
+    <row r="29" ht="50.85" customHeight="1">
       <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Dashboard</t>
@@ -2443,7 +2473,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="89.55" customHeight="1">
+    <row r="30" ht="71.7" customHeight="1">
       <c r="A30" s="7" t="inlineStr">
         <is>
           <t>Dashboard | Mis deudas</t>
@@ -2510,7 +2540,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="89.55" customHeight="1">
+    <row r="31" ht="71.7" customHeight="1">
       <c r="A31" s="7" t="inlineStr">
         <is>
           <t>Dashboard | Mis deudas</t>
@@ -2577,7 +2607,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="89.55" customHeight="1">
+    <row r="32" ht="71.7" customHeight="1">
       <c r="A32" s="7" t="inlineStr">
         <is>
           <t>Dashboard | Mis deudas</t>
@@ -2644,7 +2674,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="111.9" customHeight="1">
+    <row r="33" ht="89.55" customHeight="1">
       <c r="A33" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis deudas</t>
@@ -2711,7 +2741,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="89.55" customHeight="1">
+    <row r="34" ht="71.7" customHeight="1">
       <c r="A34" s="10" t="inlineStr">
         <is>
           <t>Dashboard | Mis deudas</t>
@@ -2778,13 +2808,13 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="105.6" customHeight="1">
+    <row r="35" ht="84.45" customHeight="1">
       <c r="A35" s="12" t="inlineStr">
         <is>
           <t>Dashboard</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>4.10</t>
         </is>
@@ -2845,13 +2875,13 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="105.6" customHeight="1">
+    <row r="36" ht="84.45" customHeight="1">
       <c r="A36" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis gastos</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
+      <c r="B36" s="13" t="inlineStr">
         <is>
           <t>4.11</t>
         </is>
@@ -2912,13 +2942,13 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="105.6" customHeight="1">
+    <row r="37" ht="84.45" customHeight="1">
       <c r="A37" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis cajitas</t>
         </is>
       </c>
-      <c r="B37" s="12" t="inlineStr">
+      <c r="B37" s="13" t="inlineStr">
         <is>
           <t>4.12</t>
         </is>
@@ -2979,13 +3009,13 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="105.6" customHeight="1">
+    <row r="38" ht="84.45" customHeight="1">
       <c r="A38" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis cajitas</t>
         </is>
       </c>
-      <c r="B38" s="12" t="inlineStr">
+      <c r="B38" s="13" t="inlineStr">
         <is>
           <t>4.13</t>
         </is>
@@ -3046,13 +3076,13 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="105.6" customHeight="1">
+    <row r="39" ht="84.45" customHeight="1">
       <c r="A39" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis ahorros</t>
         </is>
       </c>
-      <c r="B39" s="12" t="inlineStr">
+      <c r="B39" s="13" t="inlineStr">
         <is>
           <t>4.14</t>
         </is>
@@ -3113,13 +3143,13 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="105.6" customHeight="1">
+    <row r="40" ht="84.45" customHeight="1">
       <c r="A40" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis cajitas</t>
         </is>
       </c>
-      <c r="B40" s="12" t="inlineStr">
+      <c r="B40" s="13" t="inlineStr">
         <is>
           <t>4.15</t>
         </is>
@@ -3180,13 +3210,13 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="105.6" customHeight="1">
+    <row r="41" ht="84.45" customHeight="1">
       <c r="A41" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis ahorros</t>
         </is>
       </c>
-      <c r="B41" s="12" t="inlineStr">
+      <c r="B41" s="13" t="inlineStr">
         <is>
           <t>4.16</t>
         </is>
@@ -3247,13 +3277,13 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="105.6" customHeight="1">
+    <row r="42" ht="84.45" customHeight="1">
       <c r="A42" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis bolsitas</t>
         </is>
       </c>
-      <c r="B42" s="12" t="inlineStr">
+      <c r="B42" s="13" t="inlineStr">
         <is>
           <t>4.17</t>
         </is>
@@ -3314,13 +3344,13 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="105.6" customHeight="1">
+    <row r="43" ht="84.45" customHeight="1">
       <c r="A43" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis cajitas</t>
         </is>
       </c>
-      <c r="B43" s="12" t="inlineStr">
+      <c r="B43" s="13" t="inlineStr">
         <is>
           <t>4.18</t>
         </is>
@@ -3381,13 +3411,13 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="105.6" customHeight="1">
+    <row r="44" ht="84.45" customHeight="1">
       <c r="A44" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis deudas</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
+      <c r="B44" s="13" t="inlineStr">
         <is>
           <t>4.19</t>
         </is>
@@ -3448,13 +3478,13 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="105.6" customHeight="1">
+    <row r="45" ht="84.45" customHeight="1">
       <c r="A45" s="12" t="inlineStr">
         <is>
           <t>Dashboard | Mis deudas</t>
         </is>
       </c>
-      <c r="B45" s="12" t="inlineStr">
+      <c r="B45" s="13" t="inlineStr">
         <is>
           <t>4.20</t>
         </is>
@@ -3515,13 +3545,13 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="105.6" customFormat="1" customHeight="1" s="17">
+    <row r="46" ht="84.45" customFormat="1" customHeight="1" s="17">
       <c r="A46" s="15" t="inlineStr">
         <is>
           <t>Flujo de caja y ciclos de ingreso</t>
         </is>
       </c>
-      <c r="B46" s="15" t="inlineStr">
+      <c r="B46" s="22" t="inlineStr">
         <is>
           <t>5.1</t>
         </is>
@@ -3578,84 +3608,84 @@
       </c>
       <c r="M46" s="16" t="inlineStr">
         <is>
-          <t>Completo</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="105.6" customFormat="1" customHeight="1" s="17">
-      <c r="A47" s="15" t="inlineStr">
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="84.45" customFormat="1" customHeight="1" s="17">
+      <c r="A47" s="18" t="inlineStr">
         <is>
           <t>Flujo de caja y ciclos de ingreso</t>
         </is>
       </c>
-      <c r="B47" s="15" t="inlineStr">
+      <c r="B47" s="23" t="inlineStr">
         <is>
           <t>5.2</t>
         </is>
       </c>
-      <c r="C47" s="15" t="inlineStr">
-        <is>
-          <t>Registrar el monto y la fecha aproximada de cada pago</t>
-        </is>
-      </c>
-      <c r="D47" s="16" t="inlineStr">
-        <is>
-          <t>Conocer que un ingreso es quincenal no permite saber cuánto recibe la usuaria en cada pago ni cuándo lo recibe. El sistema podría asumir incorrectamente una distribución igual aunque en la vida real un pago represente, por ejemplo, 40 por ciento del ingreso y el otro 60 por ciento.</t>
-        </is>
-      </c>
-      <c r="E47" s="16" t="inlineStr">
-        <is>
-          <t>Amy debe permitir registrar cuánto dinero llega en cada pago y en qué fecha o momento aproximado del mes suele llegar, sin asumir que los pagos tienen el mismo valor.</t>
-        </is>
-      </c>
-      <c r="F47" s="16" t="inlineStr">
-        <is>
-          <t>Como una mujer que recibe diferentes montos durante el mes, quiero indicar cuánto recibo en cada pago y cuándo suele llegar, para que Amy pueda organizar mis obligaciones con el dinero que realmente tendré disponible en cada momento.</t>
-        </is>
-      </c>
-      <c r="G47" s="16" t="inlineStr">
-        <is>
-          <t>Cuando una fuente tenga más de un pago por mes, solicitar monto y fecha aproximada de cada pago. No dividir automáticamente el ingreso mensual en partes iguales. Permitir editar estos datos cuando cambie el empleo, el salario o la estructura de pagos. Para ingresos variables, permitir registrar una estimación y actualizar el monto real cuando se reciba.</t>
-        </is>
-      </c>
-      <c r="H47" s="16" t="inlineStr">
-        <is>
-          <t>Mantener el flujo simple y progresivo. Mostrar el total mensual resultante para que la usuaria pueda validar que la información registrada tiene sentido. Evitar exigir fechas exactas cuando la usuaria solo conoce un rango aproximado.</t>
-        </is>
-      </c>
-      <c r="I47" s="16" t="inlineStr">
-        <is>
-          <t>Dar a Amy información temporal suficiente para organizar el dinero de forma realista.</t>
-        </is>
-      </c>
-      <c r="J47" s="16" t="inlineStr">
-        <is>
-          <t>El plan refleja la distribución real de los ingresos dentro del mes, incluso cuando los pagos no son iguales.</t>
-        </is>
-      </c>
-      <c r="K47" s="16" t="inlineStr">
-        <is>
-          <t>Los pagos pueden tener montos diferentes, conservan su fecha aproximada y el total mensual se calcula correctamente a partir de ellos.</t>
-        </is>
-      </c>
-      <c r="L47" s="16" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="M47" s="16" t="inlineStr">
-        <is>
-          <t>Completo</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="105.6" customFormat="1" customHeight="1" s="17">
+      <c r="C47" s="18" t="inlineStr">
+        <is>
+          <t>Registrar el monto específico de cada pago y su fecha</t>
+        </is>
+      </c>
+      <c r="D47" s="19" t="inlineStr">
+        <is>
+          <t>La configuración permite indicar que un ingreso es quincenal y registrar dos fechas, pero la interfaz actual conserva un único monto general. Esto puede provocar que Amy interprete que el mismo monto llega en cada fecha o que no pueda representar casos reales en los que un pago corresponde, por ejemplo, al 40 por ciento del ingreso mensual y el otro al 60 por ciento.</t>
+        </is>
+      </c>
+      <c r="E47" s="19" t="inlineStr">
+        <is>
+          <t>Amy debe conocer el valor exacto que llega en cada fecha de pago. Una frecuencia quincenal no debe implicar que ambos pagos son iguales. La usuaria debe poder registrar de forma independiente cuánto recibe en el primer pago y cuánto recibe en el segundo.</t>
+        </is>
+      </c>
+      <c r="F47" s="19" t="inlineStr">
+        <is>
+          <t>Como una mujer que recibe dos pagos de valores diferentes durante el mes, quiero registrar cuánto dinero llega en cada fecha, para que Amy organice mi flujo usando los montos que realmente voy a recibir.</t>
+        </is>
+      </c>
+      <c r="G47" s="19" t="inlineStr">
+        <is>
+          <t>Modificar la captura de ingresos para que cada fecha tenga asociado su propio monto. Si la usuaria selecciona quincenal, permitir registrar por separado fecha del primer pago, monto del primer pago, fecha del segundo pago y monto del segundo pago. No reutilizar el ingreso mensual total como valor del próximo pago. Mostrar el total mensual calculado como referencia y permitir editar cada pago individualmente. Aplicar la misma lógica a otras frecuencias con múltiples pagos.</t>
+        </is>
+      </c>
+      <c r="H47" s="19" t="inlineStr">
+        <is>
+          <t>Evitar formularios ambiguos donde exista un solo campo Monto junto a varias fechas. La relación entre fecha y valor debe ser visualmente evidente. El total mensual debe ser una consecuencia de los pagos registrados, no una suposición sobre cómo se distribuyen.</t>
+        </is>
+      </c>
+      <c r="I47" s="19" t="inlineStr">
+        <is>
+          <t>Representar correctamente ingresos que no se distribuyen de forma uniforme y mejorar la precisión de todo el flujo de caja.</t>
+        </is>
+      </c>
+      <c r="J47" s="19" t="inlineStr">
+        <is>
+          <t>Amy sabe exactamente cuánto dinero llegará en cada fecha y puede construir recomendaciones diferentes para cada pago.</t>
+        </is>
+      </c>
+      <c r="K47" s="19" t="inlineStr">
+        <is>
+          <t>Cada fecha de ingreso tiene un monto propio, el próximo ingreso muestra el valor correspondiente a esa fecha y casos como 40 por ciento y 60 por ciento se calculan correctamente.</t>
+        </is>
+      </c>
+      <c r="L47" s="19" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M47" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="84.45" customFormat="1" customHeight="1" s="17">
       <c r="A48" s="15" t="inlineStr">
         <is>
           <t>Flujo de caja y ciclos de ingreso</t>
         </is>
       </c>
-      <c r="B48" s="15" t="inlineStr">
+      <c r="B48" s="22" t="inlineStr">
         <is>
           <t>5.3</t>
         </is>
@@ -3712,84 +3742,84 @@
       </c>
       <c r="M48" s="16" t="inlineStr">
         <is>
-          <t>Completo</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="105.6" customFormat="1" customHeight="1" s="17">
-      <c r="A49" s="15" t="inlineStr">
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="84.45" customFormat="1" customHeight="1" s="17">
+      <c r="A49" s="18" t="inlineStr">
         <is>
           <t>Flujo de caja y ciclos de ingreso</t>
         </is>
       </c>
-      <c r="B49" s="15" t="inlineStr">
+      <c r="B49" s="23" t="inlineStr">
         <is>
           <t>5.4</t>
         </is>
       </c>
-      <c r="C49" s="15" t="inlineStr">
-        <is>
-          <t>Detectar falta de liquidez entre un ingreso y el siguiente</t>
-        </is>
-      </c>
-      <c r="D49" s="16" t="inlineStr">
-        <is>
-          <t>Una usuaria puede tener capacidad financiera positiva al finalizar el mes y aun así quedarse prácticamente sin dinero durante varios días porque sus obligaciones se concentran antes de uno de sus pagos. El cálculo mensual puede mostrar dinero disponible y ocultar este problema.</t>
-        </is>
-      </c>
-      <c r="E49" s="16" t="inlineStr">
-        <is>
-          <t>Antes de recomendar ahorro o mostrar dinero libre, Amy debe revisar cada periodo entre ingresos y detectar si la usuaria tendrá suficiente dinero para cubrir obligaciones y gastos necesarios hasta recibir el siguiente pago.</t>
-        </is>
-      </c>
-      <c r="F49" s="16" t="inlineStr">
-        <is>
-          <t>Como una mujer cuyos ingresos mensuales sí alcanzan pero están distribuidos de forma desigual, quiero que Amy detecte cuando una parte del mes queda demasiado ajustada, para no creer que tengo dinero disponible cuando todavía necesito cubrir los días antes de mi próximo pago.</t>
-        </is>
-      </c>
-      <c r="G49" s="16" t="inlineStr">
-        <is>
-          <t>Construir periodos de flujo de caja desde cada ingreso hasta el siguiente. Para cada periodo calcular dinero inicial, ingresos recibidos, obligaciones que vencen durante ese intervalo, reservas ya asignadas y monto restante para los gastos necesarios del periodo. Si el resultado deja a la usuaria sin liquidez suficiente, identificar el desbalance antes de calcular capacidad de ahorro. No clasificar automáticamente el caso como falta de ingresos mensuales si el problema es temporal.</t>
-        </is>
-      </c>
-      <c r="H49" s="16" t="inlineStr">
-        <is>
-          <t>Comunicar el hallazgo sin alarmar ni culpabilizar. Explicar la diferencia entre que el mes alcance y que el dinero esté disponible en el momento correcto. Evitar mostrar como libre dinero que ya se necesita para un periodo futuro.</t>
-        </is>
-      </c>
-      <c r="I49" s="16" t="inlineStr">
-        <is>
-          <t>Evitar recomendaciones de ahorro que comprometan la capacidad de la usuaria para llegar a su siguiente ingreso.</t>
-        </is>
-      </c>
-      <c r="J49" s="16" t="inlineStr">
-        <is>
-          <t>Amy distingue entre capacidad mensual y liquidez dentro del mes y puede intervenir antes de que aparezca un periodo sin dinero.</t>
-        </is>
-      </c>
-      <c r="K49" s="16" t="inlineStr">
-        <is>
-          <t>El sistema identifica periodos con insuficiente liquidez aunque el balance mensual sea positivo y no recomienda como disponible el dinero necesario para cubrirlos.</t>
-        </is>
-      </c>
-      <c r="L49" s="16" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="M49" s="16" t="inlineStr">
-        <is>
-          <t>Completo</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="105.6" customFormat="1" customHeight="1" s="17">
+      <c r="C49" s="18" t="inlineStr">
+        <is>
+          <t>Detectar y explicar periodos que quedarán ajustados</t>
+        </is>
+      </c>
+      <c r="D49" s="19" t="inlineStr">
+        <is>
+          <t>El sistema puede calcular el periodo entre ingresos, pero la experiencia actual se limita principalmente a informar si existen pagos antes del próximo ingreso y cuánto dinero quedará. Esto no genera suficiente valor cuando Amy detecta que una parte del mes quedará demasiado ajustada.</t>
+        </is>
+      </c>
+      <c r="E49" s="19" t="inlineStr">
+        <is>
+          <t>Cuando Amy detecte poca liquidez antes de un ingreso futuro, debe convertir ese hallazgo en una recomendación concreta. Debe explicar qué periodo queda ajustado, cuánto dinero faltaría o sería recomendable proteger y desde qué ingreso más holgado puede prepararse.</t>
+        </is>
+      </c>
+      <c r="F49" s="19" t="inlineStr">
+        <is>
+          <t>Como una mujer cuyos ingresos mensuales sí alcanzan pero no están distribuidos de forma equilibrada, quiero que Amy me avise antes de que llegue una quincena difícil y me diga cómo prepararme, para no descubrir el problema cuando ya me quede sin dinero.</t>
+        </is>
+      </c>
+      <c r="G49" s="19" t="inlineStr">
+        <is>
+          <t>Analizar cada intervalo entre ingresos y comparar el dinero disponible con obligaciones y necesidades del periodo. Cuando exista un desbalance, mostrar un insight visible de Amy con el problema y la acción recomendada. Ejemplo conceptual: 'Tu primera quincena queda muy ajustada. Cuando recibas tu segundo pago, deja $X preparados para complementar la siguiente'. El insight debe actualizarse cuando cambien ingresos, saldo u obligaciones.</t>
+        </is>
+      </c>
+      <c r="H49" s="19" t="inlineStr">
+        <is>
+          <t>El mensaje debe enfocarse en anticipación, no en alarma. Evitar mostrar únicamente cifras o estados como 'llegas con $X'. Amy debe explicar por qué importa y qué debe hacer la usuaria con esa información.</t>
+        </is>
+      </c>
+      <c r="I49" s="19" t="inlineStr">
+        <is>
+          <t>Convertir el análisis de flujo de caja en prevención activa y reducir periodos de falta de liquidez.</t>
+        </is>
+      </c>
+      <c r="J49" s="19" t="inlineStr">
+        <is>
+          <t>La usuaria descubre los desbalances antes de vivirlos y recibe una acción concreta para corregirlos.</t>
+        </is>
+      </c>
+      <c r="K49" s="19" t="inlineStr">
+        <is>
+          <t>Cuando existe un periodo ajustado, Amy lo identifica, cuantifica la necesidad y presenta una recomendación accionable antes de que ocurra.</t>
+        </is>
+      </c>
+      <c r="L49" s="19" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M49" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="84.45" customFormat="1" customHeight="1" s="17">
       <c r="A50" s="15" t="inlineStr">
         <is>
           <t>Flujo de caja y ciclos de ingreso</t>
         </is>
       </c>
-      <c r="B50" s="15" t="inlineStr">
+      <c r="B50" s="22" t="inlineStr">
         <is>
           <t>5.5</t>
         </is>
@@ -3846,17 +3876,17 @@
       </c>
       <c r="M50" s="16" t="inlineStr">
         <is>
-          <t>Completo</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="105.6" customFormat="1" customHeight="1" s="17">
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="84.45" customFormat="1" customHeight="1" s="17">
       <c r="A51" s="15" t="inlineStr">
         <is>
           <t>Flujo de caja y ciclos de ingreso</t>
         </is>
       </c>
-      <c r="B51" s="15" t="inlineStr">
+      <c r="B51" s="22" t="inlineStr">
         <is>
           <t>5.6</t>
         </is>
@@ -3913,151 +3943,151 @@
       </c>
       <c r="M51" s="16" t="inlineStr">
         <is>
-          <t>Completo</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="105.6" customFormat="1" customHeight="1" s="17">
-      <c r="A52" s="15" t="inlineStr">
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="84.45" customFormat="1" customHeight="1" s="17">
+      <c r="A52" s="18" t="inlineStr">
         <is>
           <t>Flujo de caja y ciclos de ingreso</t>
         </is>
       </c>
-      <c r="B52" s="15" t="inlineStr">
+      <c r="B52" s="23" t="inlineStr">
         <is>
           <t>5.7</t>
         </is>
       </c>
-      <c r="C52" s="15" t="inlineStr">
-        <is>
-          <t>Mostrar en el dashboard el plan hasta el próximo ingreso</t>
-        </is>
-      </c>
-      <c r="D52" s="16" t="inlineStr">
-        <is>
-          <t>El dashboard se organiza principalmente alrededor del mes, pero una usuaria que recibe varios pagos necesita saber qué debe hacer con el dinero disponible ahora y qué debe cubrir antes de recibir el siguiente ingreso.</t>
-        </is>
-      </c>
-      <c r="E52" s="16" t="inlineStr">
-        <is>
-          <t>Además de conservar la visión mensual, el dashboard debe mostrar un plan sencillo para el periodo actual con el próximo ingreso, las obligaciones que deben cubrirse antes de esa fecha, el dinero reservado y el monto que realmente puede utilizarse.</t>
-        </is>
-      </c>
-      <c r="F52" s="16" t="inlineStr">
-        <is>
-          <t>Como una mujer que recibe varios pagos durante el mes, quiero ver qué debo cubrir hasta mi próximo ingreso, para tomar decisiones con el dinero que tengo hoy sin perder de vista mi plan mensual.</t>
-        </is>
-      </c>
-      <c r="G52" s="16" t="inlineStr">
-        <is>
-          <t>Crear un bloque de periodo actual dentro del dashboard para usuarias cuya frecuencia de ingreso lo requiera. Mostrar fecha aproximada del próximo ingreso, obligaciones pendientes antes de esa fecha, reservas asignadas y dinero disponible para ese periodo. Al llegar un nuevo ingreso, avanzar al siguiente periodo y recalcular la información. Mantener la visión mensual como contexto general.</t>
-        </is>
-      </c>
-      <c r="H52" s="16" t="inlineStr">
-        <is>
-          <t>Evitar duplicar todo el dashboard. La vista del periodo debe responder una pregunta concreta: qué necesito hacer con mi dinero hasta que vuelva a recibir ingresos. Mantener jerarquía visual clara entre mes y periodo actual.</t>
-        </is>
-      </c>
-      <c r="I52" s="16" t="inlineStr">
-        <is>
-          <t>Convertir el dashboard en una herramienta útil para decisiones cotidianas y aumentar la frecuencia de uso de Amy.</t>
-        </is>
-      </c>
-      <c r="J52" s="16" t="inlineStr">
-        <is>
-          <t>La usuaria entiende su mes completo y al mismo tiempo sabe qué debe hacer con el dinero disponible hasta el próximo pago.</t>
-        </is>
-      </c>
-      <c r="K52" s="16" t="inlineStr">
-        <is>
-          <t>El dashboard muestra el periodo vigente, el siguiente ingreso y las obligaciones que deben cubrirse antes de recibirlo con datos consistentes con el plan mensual.</t>
-        </is>
-      </c>
-      <c r="L52" s="16" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="M52" s="16" t="inlineStr">
-        <is>
-          <t>Completo</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="105.6" customFormat="1" customHeight="1" s="17">
-      <c r="A53" s="15" t="inlineStr">
+      <c r="C52" s="18" t="inlineStr">
+        <is>
+          <t>Convertir el plan hasta el próximo ingreso en la información principal</t>
+        </is>
+      </c>
+      <c r="D52" s="19" t="inlineStr">
+        <is>
+          <t>La sección actual da gran protagonismo a campos de captura y listas de datos. El bloque 'Tu plan hasta el próximo ingreso' muestra el siguiente pago y si existen obligaciones, pero todavía obliga a la usuaria a interpretar cuánto puede usar y qué debería hacer ahora.</t>
+        </is>
+      </c>
+      <c r="E52" s="19" t="inlineStr">
+        <is>
+          <t>Al entrar a la sección, la primera información debe ser el análisis de Amy. El plan debe responder inmediatamente cuánto dinero tiene hoy, cuánto necesita proteger antes del próximo ingreso, cuánto puede usar con tranquilidad y cuál es la siguiente acción recomendada.</t>
+        </is>
+      </c>
+      <c r="F52" s="19" t="inlineStr">
+        <is>
+          <t>Como una mujer que ya le contó a Amy cuándo recibe dinero y cuándo tiene que pagar, quiero que Amy transforme esos datos en un plan claro para los próximos días, para no tener que hacer yo misma los cálculos.</t>
+        </is>
+      </c>
+      <c r="G52" s="19" t="inlineStr">
+        <is>
+          <t>Reestructurar la jerarquía de la sección para que el plan accionable aparezca antes de los formularios de configuración. El bloque principal debe mostrar como mínimo dinero disponible hoy, dinero con destino antes del próximo ingreso, dinero realmente utilizable y próxima acción. Si no existen obligaciones antes del próximo ingreso, Amy debe igualmente explicar qué parte puede utilizarse y si existe dinero que deba reservarse para un periodo posterior. Recalcular ante cualquier cambio relevante.</t>
+        </is>
+      </c>
+      <c r="H52" s="19" t="inlineStr">
+        <is>
+          <t>La primera pantalla visible debe entregar valor y no pedir trabajo adicional. Evitar devolver únicamente datos que la usuaria ya ingresó. La frase principal debe responder qué puede hacer con su dinero ahora.</t>
+        </is>
+      </c>
+      <c r="I52" s="19" t="inlineStr">
+        <is>
+          <t>Demostrar el valor de Amy como guía financiera y no solo como repositorio de información.</t>
+        </is>
+      </c>
+      <c r="J52" s="19" t="inlineStr">
+        <is>
+          <t>La usuaria entiende qué hacer con su dinero actual en pocos segundos y no necesita interpretar manualmente ingresos y pagos.</t>
+        </is>
+      </c>
+      <c r="K52" s="19" t="inlineStr">
+        <is>
+          <t>Sin hacer scroll ni cálculos propios, la usuaria puede identificar cuánto puede usar, cuánto debe proteger y cuál es su siguiente acción.</t>
+        </is>
+      </c>
+      <c r="L52" s="19" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M52" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="84.45" customFormat="1" customHeight="1" s="17">
+      <c r="A53" s="18" t="inlineStr">
         <is>
           <t>Flujo de caja y ciclos de ingreso</t>
         </is>
       </c>
-      <c r="B53" s="15" t="inlineStr">
+      <c r="B53" s="23" t="inlineStr">
         <is>
           <t>5.8</t>
         </is>
       </c>
-      <c r="C53" s="15" t="inlineStr">
-        <is>
-          <t>Diferenciar saldo en cuenta de dinero realmente disponible</t>
-        </is>
-      </c>
-      <c r="D53" s="16" t="inlineStr">
-        <is>
-          <t>Una usuaria puede ver un saldo alto en su cuenta después de recibir un pago, pero una parte de ese dinero puede estar destinada a obligaciones o a complementar el siguiente periodo. Mostrar todo el saldo como disponible puede llevarla a gastar o ahorrar dinero que ya tiene un propósito.</t>
-        </is>
-      </c>
-      <c r="E53" s="16" t="inlineStr">
-        <is>
-          <t>Amy debe separar conceptualmente el dinero que existe en la cuenta del dinero que realmente está libre para decisiones nuevas después de proteger obligaciones y reservas.</t>
-        </is>
-      </c>
-      <c r="F53" s="16" t="inlineStr">
-        <is>
-          <t>Como una mujer que acaba de recibir mi salario, quiero saber cuánto de ese dinero realmente puedo usar, para no confundir tener dinero en la cuenta con tener dinero libre.</t>
-        </is>
-      </c>
-      <c r="G53" s="16" t="inlineStr">
-        <is>
-          <t>Actualizar la lógica de Dinero disponible para excluir obligaciones pendientes, cajitas, compromisos confirmados y reservas necesarias para periodos futuros según las reglas vigentes del producto. Cuando exista dinero reservado para el siguiente periodo, mostrarlo de forma separada y explicar su propósito. Todos los módulos que utilicen Dinero disponible deben consumir la misma lógica central.</t>
-        </is>
-      </c>
-      <c r="H53" s="16" t="inlineStr">
-        <is>
-          <t>Usar términos muy claros y consistentes. La usuaria debe poder entender por qué su saldo bancario puede ser mayor que el monto que Amy considera disponible sin sentir que el dinero desapareció.</t>
-        </is>
-      </c>
-      <c r="I53" s="16" t="inlineStr">
-        <is>
-          <t>Evitar decisiones basadas en una falsa sensación de liquidez y fortalecer la confianza en los cálculos de Amy.</t>
-        </is>
-      </c>
-      <c r="J53" s="16" t="inlineStr">
-        <is>
-          <t>La usuaria sabe qué parte de su dinero tiene destino y qué parte puede utilizar para nuevas decisiones.</t>
-        </is>
-      </c>
-      <c r="K53" s="16" t="inlineStr">
-        <is>
-          <t>Dinero disponible excluye correctamente las reservas y obligaciones comprometidas y la diferencia puede explicarse desde el dashboard.</t>
-        </is>
-      </c>
-      <c r="L53" s="16" t="inlineStr">
-        <is>
-          <t>Alta</t>
-        </is>
-      </c>
-      <c r="M53" s="16" t="inlineStr">
-        <is>
-          <t>Completo</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="105.6" customFormat="1" customHeight="1" s="17">
+      <c r="C53" s="18" t="inlineStr">
+        <is>
+          <t>Mostrar dinero realmente utilizable y explicar qué parte ya tiene destino</t>
+        </is>
+      </c>
+      <c r="D53" s="19" t="inlineStr">
+        <is>
+          <t>La pantalla pregunta cuánto tiene hoy la usuaria en su cuenta, pero el saldo bancario por sí solo no representa cuánto puede gastar. Parte de ese dinero puede estar comprometida para pagos próximos o para equilibrar un periodo futuro.</t>
+        </is>
+      </c>
+      <c r="E53" s="19" t="inlineStr">
+        <is>
+          <t>Amy debe convertir el saldo actual en una cifra útil. Debe separar de forma visible cuánto dinero existe hoy, cuánto ya tiene un destino y cuánto puede utilizar la usuaria con tranquilidad hasta su próximo ingreso.</t>
+        </is>
+      </c>
+      <c r="F53" s="19" t="inlineStr">
+        <is>
+          <t>Como una mujer que ve un saldo en mi cuenta pero sé que parte de ese dinero ya está comprometido, quiero que Amy me diga cuánto puedo usar realmente, para no gastar dinero que voy a necesitar después.</t>
+        </is>
+      </c>
+      <c r="G53" s="19" t="inlineStr">
+        <is>
+          <t>Tomar el saldo actual como punto de partida y descontar obligaciones pendientes antes del próximo ingreso, reservas necesarias para periodos futuros y demás compromisos que según la lógica central ya tengan destino. Mostrar el resultado como 'Puedes usar $X con tranquilidad hasta tu próximo ingreso' o una formulación equivalente. Permitir ver un desglose sencillo de por qué el saldo en cuenta y el dinero utilizable son diferentes.</t>
+        </is>
+      </c>
+      <c r="H53" s="19" t="inlineStr">
+        <is>
+          <t>No presentar el saldo actual como la cifra protagonista si no es accionable. La usuaria debe entender la diferencia sin conocer conceptos de flujo de caja. Mantener una única definición de dinero disponible en todos los módulos.</t>
+        </is>
+      </c>
+      <c r="I53" s="19" t="inlineStr">
+        <is>
+          <t>Evitar una falsa sensación de liquidez y mejorar la confianza en las recomendaciones de Amy.</t>
+        </is>
+      </c>
+      <c r="J53" s="19" t="inlineStr">
+        <is>
+          <t>La usuaria distingue claramente entre dinero que existe en la cuenta y dinero que realmente puede utilizar.</t>
+        </is>
+      </c>
+      <c r="K53" s="19" t="inlineStr">
+        <is>
+          <t>El sistema calcula una cifra utilizable después de compromisos y reservas, la muestra de forma protagonista y permite entender su composición.</t>
+        </is>
+      </c>
+      <c r="L53" s="19" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M53" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="84.45" customFormat="1" customHeight="1" s="17">
       <c r="A54" s="15" t="inlineStr">
         <is>
           <t>Flujo de caja y ciclos de ingreso</t>
         </is>
       </c>
-      <c r="B54" s="15" t="inlineStr">
+      <c r="B54" s="22" t="inlineStr">
         <is>
           <t>5.9</t>
         </is>
@@ -4114,17 +4144,17 @@
       </c>
       <c r="M54" s="16" t="inlineStr">
         <is>
-          <t>Completo</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="105.6" customFormat="1" customHeight="1" s="17">
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="84.45" customFormat="1" customHeight="1" s="17">
       <c r="A55" s="15" t="inlineStr">
         <is>
           <t>Flujo de caja y ciclos de ingreso</t>
         </is>
       </c>
-      <c r="B55" s="15" t="inlineStr">
+      <c r="B55" s="22" t="inlineStr">
         <is>
           <t>5.10</t>
         </is>
@@ -4181,11 +4211,481 @@
       </c>
       <c r="M55" s="16" t="inlineStr">
         <is>
-          <t>Completo</t>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="84.45" customFormat="1" customHeight="1" s="17">
+      <c r="A56" s="18" t="inlineStr">
+        <is>
+          <t>Flujo de caja y ciclos de ingreso</t>
+        </is>
+      </c>
+      <c r="B56" s="23" t="inlineStr">
+        <is>
+          <t>5.11</t>
+        </is>
+      </c>
+      <c r="C56" s="18" t="inlineStr">
+        <is>
+          <t>Distribuir cada ingreso entre sus destinos</t>
+        </is>
+      </c>
+      <c r="D56" s="19" t="inlineStr">
+        <is>
+          <t>La sección muestra cuándo llega el dinero y cuándo salen algunos pagos, pero todavía no le dice a la usuaria cómo repartir cada ingreso cuando lo reciba. La usuaria sigue teniendo que decidir por su cuenta cuánto separar para obligaciones, cuánto reservar para el siguiente periodo, cuánto destinar al ahorro y cuánto puede utilizar.</t>
+        </is>
+      </c>
+      <c r="E56" s="19" t="inlineStr">
+        <is>
+          <t>Para cada ingreso futuro, Amy debe construir una distribución concreta del dinero. Cuando llegue un pago, la usuaria debe poder ver qué parte corresponde a obligaciones, qué parte debe reservarse para otro periodo, qué parte puede ir a ahorro y qué parte queda realmente disponible.</t>
+        </is>
+      </c>
+      <c r="F56" s="19" t="inlineStr">
+        <is>
+          <t>Como una mujer que recibe varios pagos durante el mes, quiero que Amy me diga cómo repartir cada uno cuando llegue, para no tener que reconstruir mi presupuesto cada quincena.</t>
+        </is>
+      </c>
+      <c r="G56" s="19" t="inlineStr">
+        <is>
+          <t>Crear un plan por ingreso. Cada pago debe mostrar su fecha, monto esperado y distribución recomendada según la información financiera vigente. La suma de los destinos no puede superar el ingreso disponible para ese periodo. Si una categoría no aplica, no mostrarla. Cuando cambien ingresos, obligaciones, reservas o ahorro, recalcular la distribución. La lógica debe distinguir dinero para obligaciones inmediatas, reserva para periodos futuros, ahorro planificado y dinero utilizable.</t>
+        </is>
+      </c>
+      <c r="H56" s="19" t="inlineStr">
+        <is>
+          <t>Presentar la distribución como un plan simple, no como una tabla contable. Priorizar frases accionables como 'De este pago, separa $X para...' y mantener visible el monto que queda después de cada asignación.</t>
+        </is>
+      </c>
+      <c r="I56" s="19" t="inlineStr">
+        <is>
+          <t>Transformar cada ingreso en una decisión guiada y aumentar el valor práctico de Amy en el momento en que la usuaria recibe dinero.</t>
+        </is>
+      </c>
+      <c r="J56" s="19" t="inlineStr">
+        <is>
+          <t>La usuaria sabe exactamente qué hacer con cada pago y no necesita crear manualmente una distribución fuera de Finance BFF.</t>
+        </is>
+      </c>
+      <c r="K56" s="19" t="inlineStr">
+        <is>
+          <t>Cada ingreso tiene una distribución coherente, los destinos suman correctamente y la usuaria puede identificar cuánto separar y cuánto queda libre.</t>
+        </is>
+      </c>
+      <c r="L56" s="19" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M56" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="84.45" customFormat="1" customHeight="1" s="17">
+      <c r="A57" s="18" t="inlineStr">
+        <is>
+          <t>Flujo de caja y ciclos de ingreso</t>
+        </is>
+      </c>
+      <c r="B57" s="23" t="inlineStr">
+        <is>
+          <t>5.12</t>
+        </is>
+      </c>
+      <c r="C57" s="18" t="inlineStr">
+        <is>
+          <t>Mostrar una línea de tiempo sencilla de próximos ingresos y obligaciones</t>
+        </is>
+      </c>
+      <c r="D57" s="19" t="inlineStr">
+        <is>
+          <t>Los ingresos y pagos aparecen actualmente como listas separadas. Para comprender qué ocurre primero, la usuaria debe comparar mentalmente fechas entre diferentes bloques de la página.</t>
+        </is>
+      </c>
+      <c r="E57" s="19" t="inlineStr">
+        <is>
+          <t>Amy debe mostrar de forma visual y cronológica los próximos movimientos relevantes para que la usuaria pueda entender cómo se comportará su dinero durante las siguientes semanas.</t>
+        </is>
+      </c>
+      <c r="F57" s="19" t="inlineStr">
+        <is>
+          <t>Como una mujer que recibe y paga dinero en diferentes fechas, quiero ver mis próximos ingresos y obligaciones en orden, para entender rápidamente qué ocurre antes de mi siguiente pago y qué debo preparar.</t>
+        </is>
+      </c>
+      <c r="G57" s="19" t="inlineStr">
+        <is>
+          <t>Crear una línea de tiempo compacta que combine próximos ingresos y obligaciones relevantes en orden cronológico. Diferenciar claramente entradas y salidas sin recargar la interfaz. Mostrar monto y fecha cuando estén disponibles. Permitir que la usuaria identifique visualmente los periodos entre un ingreso y el siguiente. La línea de tiempo debe alimentarse de los mismos datos existentes y no requerir una segunda captura.</t>
+        </is>
+      </c>
+      <c r="H57" s="19" t="inlineStr">
+        <is>
+          <t>Debe servir para comprensión, no convertirse en un calendario complejo. Priorizar los movimientos que afectan decisiones próximas y permitir ampliar detalles solo cuando sea necesario.</t>
+        </is>
+      </c>
+      <c r="I57" s="19" t="inlineStr">
+        <is>
+          <t>Reducir esfuerzo cognitivo y hacer visible el flujo temporal que Amy está utilizando para sus recomendaciones.</t>
+        </is>
+      </c>
+      <c r="J57" s="19" t="inlineStr">
+        <is>
+          <t>La usuaria comprende de un vistazo qué dinero entra, qué obligaciones salen y en qué orden ocurren.</t>
+        </is>
+      </c>
+      <c r="K57" s="19" t="inlineStr">
+        <is>
+          <t>Los movimientos se presentan cronológicamente y coinciden con los datos usados por el cálculo del plan.</t>
+        </is>
+      </c>
+      <c r="L57" s="19" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="M57" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="84.45" customFormat="1" customHeight="1" s="17">
+      <c r="A58" s="18" t="inlineStr">
+        <is>
+          <t>Flujo de caja y ciclos de ingreso</t>
+        </is>
+      </c>
+      <c r="B58" s="23" t="inlineStr">
+        <is>
+          <t>5.13</t>
+        </is>
+      </c>
+      <c r="C58" s="18" t="inlineStr">
+        <is>
+          <t>Mover la configuración de ingresos y pagos a un nivel secundario</t>
+        </is>
+      </c>
+      <c r="D58" s="19" t="inlineStr">
+        <is>
+          <t>En la experiencia actual, los formularios para agregar ingresos y pagos ocupan gran parte de la pantalla principal. Esto hace que la sección se sienta como una herramienta de captura de datos y reduce el protagonismo del análisis de Amy.</t>
+        </is>
+      </c>
+      <c r="E58" s="19" t="inlineStr">
+        <is>
+          <t>La pantalla principal debe estar dedicada al plan y a las recomendaciones. Los datos de ingresos y obligaciones deben seguir siendo fáciles de consultar y editar, pero como configuración secundaria.</t>
+        </is>
+      </c>
+      <c r="F58" s="19" t="inlineStr">
+        <is>
+          <t>Como una usuaria que ya configuró mis ingresos y pagos, quiero ver primero mi plan y abrir la edición solo cuando necesite cambiar algo, para que la sección me ayude a tomar decisiones en vez de mostrarme formularios todo el tiempo.</t>
+        </is>
+      </c>
+      <c r="G58" s="19" t="inlineStr">
+        <is>
+          <t>Convertir los bloques de configuración en secciones resumidas y expandibles o en una vista secundaria de edición. En estado cerrado mostrar información útil como cantidad de ingresos registrados, próximo ingreso y cantidad de pagos fijos. Al seleccionar Editar o Agregar, desplegar los campos correspondientes. Después de guardar, regresar al estado resumido y recalcular el plan.</t>
+        </is>
+      </c>
+      <c r="H58" s="19" t="inlineStr">
+        <is>
+          <t>No esconder información esencial para entender el plan. La configuración debe estar disponible sin dominar visualmente la página. Evitar mostrar campos vacíos permanentemente cuando la usuaria no está realizando una edición.</t>
+        </is>
+      </c>
+      <c r="I58" s="19" t="inlineStr">
+        <is>
+          <t>Dar protagonismo al valor generado por Amy y reducir la sensación de estar diligenciando un Excel.</t>
+        </is>
+      </c>
+      <c r="J58" s="19" t="inlineStr">
+        <is>
+          <t>La usuaria entra para consultar su plan y solo interactúa con formularios cuando necesita actualizar información.</t>
+        </is>
+      </c>
+      <c r="K58" s="19" t="inlineStr">
+        <is>
+          <t>Los formularios no dominan la vista inicial, pueden abrirse bajo demanda y cualquier edición actualiza inmediatamente el análisis.</t>
+        </is>
+      </c>
+      <c r="L58" s="19" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M58" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="84.45" customFormat="1" customHeight="1" s="17">
+      <c r="A59" s="18" t="inlineStr">
+        <is>
+          <t>Flujo de caja y ciclos de ingreso</t>
+        </is>
+      </c>
+      <c r="B59" s="23" t="inlineStr">
+        <is>
+          <t>5.14</t>
+        </is>
+      </c>
+      <c r="C59" s="18" t="inlineStr">
+        <is>
+          <t>Renombrar Mis ciclos como Mi plan de ingresos</t>
+        </is>
+      </c>
+      <c r="D59" s="19" t="inlineStr">
+        <is>
+          <t>El menú utiliza el nombre 'Mis ciclos'. Aunque describe la lógica interna del producto, no comunica inmediatamente qué encontrará allí una usuaria que no conoce el concepto de ciclos de ingreso.</t>
+        </is>
+      </c>
+      <c r="E59" s="19" t="inlineStr">
+        <is>
+          <t>La sección debe llamarse 'Mi plan de ingresos' para comunicar de manera más cercana que allí Amy organiza cuándo llega el dinero, qué debe cubrirse entre un ingreso y el siguiente y cómo prepararse para los próximos pagos.</t>
+        </is>
+      </c>
+      <c r="F59" s="19" t="inlineStr">
+        <is>
+          <t>Como una usuaria que navega por Finance BFF, quiero reconocer por el nombre del menú que esta sección me ayuda a organizar mis ingresos durante el mes, para encontrarla sin tener que aprender terminología interna del producto.</t>
+        </is>
+      </c>
+      <c r="G59" s="19" t="inlineStr">
+        <is>
+          <t>Reemplazar 'Mis ciclos' por 'Mi plan de ingresos' en el menú lateral, título de la página y cualquier referencia interna visible para la usuaria. Mantener 'Flujo de caja y ciclos de ingreso' únicamente como nombre interno del Epic si resulta útil para producto y desarrollo.</t>
+        </is>
+      </c>
+      <c r="H59" s="19" t="inlineStr">
+        <is>
+          <t>Usar siempre lenguaje cotidiano frente a la usuaria. Evitar expresiones técnicas como flujo de caja o ciclos de ingreso como título principal. El nombre debe convivir claramente con Mis finanzas, Ingresos y las demás secciones del menú.</t>
+        </is>
+      </c>
+      <c r="I59" s="19" t="inlineStr">
+        <is>
+          <t>Mejorar descubribilidad, comprensión de navegación y percepción de cercanía de Finance BFF.</t>
+        </is>
+      </c>
+      <c r="J59" s="19" t="inlineStr">
+        <is>
+          <t>La usuaria entiende por el nombre que la sección organiza cómo recibe y utiliza sus ingresos a lo largo del mes.</t>
+        </is>
+      </c>
+      <c r="K59" s="19" t="inlineStr">
+        <is>
+          <t>'Mi plan de ingresos' aparece de forma consistente en toda la interfaz y ya no se muestra 'Mis ciclos' como nombre de la sección.</t>
+        </is>
+      </c>
+      <c r="L59" s="19" t="inlineStr">
+        <is>
+          <t>Media</t>
+        </is>
+      </c>
+      <c r="M59" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="84.45" customFormat="1" customHeight="1" s="17">
+      <c r="A60" s="18" t="inlineStr">
+        <is>
+          <t>Flujo de caja y ciclos de ingreso</t>
+        </is>
+      </c>
+      <c r="B60" s="23" t="inlineStr">
+        <is>
+          <t>5.15</t>
+        </is>
+      </c>
+      <c r="C60" s="18" t="inlineStr">
+        <is>
+          <t>Explicar qué es Mi plan de ingresos y para qué sirve</t>
+        </is>
+      </c>
+      <c r="D60" s="19" t="inlineStr">
+        <is>
+          <t>La sección empieza directamente con datos y cálculos, por lo que una usuaria puede no entender por qué existe esta vista ni qué diferencia tiene frente a Mis finanzas o Ingresos. Sin contexto, la funcionalidad puede sentirse como otra pantalla para registrar números.</t>
+        </is>
+      </c>
+      <c r="E60" s="19" t="inlineStr">
+        <is>
+          <t>Al entrar a Mi plan de ingresos, Amy debe explicar en pocas palabras que esta sección organiza el dinero según cuándo llega y cuándo se necesita, con el objetivo de ayudar a la usuaria a llegar tranquila a su próximo ingreso y anticipar periodos que podrían quedar ajustados.</t>
+        </is>
+      </c>
+      <c r="F60" s="19" t="inlineStr">
+        <is>
+          <t>Como una mujer que entra por primera vez a Mi plan de ingresos, quiero entender inmediatamente para qué sirve esta sección y qué hará Amy con mis datos, para saber por qué vale la pena usarla.</t>
+        </is>
+      </c>
+      <c r="G60" s="19" t="inlineStr">
+        <is>
+          <t>Incluir una introducción breve y visible cerca del título de la sección. Debe explicar el beneficio antes de entrar en configuraciones o cálculos. Conceptualmente debe comunicar: 'Aquí Amy organiza tu dinero según cuándo lo recibes y cuándo tienes que usarlo, para ayudarte a llegar tranquila a tu próximo pago'. El copy final puede adaptarse al tono de Finance BFF, pero debe conservar esa idea. Evitar repetir explicaciones largas en cada visita si ya no aportan valor.</t>
+        </is>
+      </c>
+      <c r="H60" s="19" t="inlineStr">
+        <is>
+          <t>La explicación debe ser corta, humana y centrada en el beneficio. No usar términos como flujo de caja, liquidez o ciclo financiero como requisito para comprender la sección. Debe diferenciarse claramente de Mis finanzas, que muestra la fotografía general.</t>
+        </is>
+      </c>
+      <c r="I60" s="19" t="inlineStr">
+        <is>
+          <t>Aumentar comprensión y percepción de valor de una funcionalidad nueva para la usuaria.</t>
+        </is>
+      </c>
+      <c r="J60" s="19" t="inlineStr">
+        <is>
+          <t>La usuaria entiende por qué existe Mi plan de ingresos y qué problema le ayuda a resolver antes de interactuar con los datos.</t>
+        </is>
+      </c>
+      <c r="K60" s="19" t="inlineStr">
+        <is>
+          <t>La sección incluye una explicación visible y breve que comunica propósito, beneficio y relación entre fechas de ingreso y uso del dinero.</t>
+        </is>
+      </c>
+      <c r="L60" s="19" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M60" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="84.45" customFormat="1" customHeight="1" s="17">
+      <c r="A61" s="18" t="inlineStr">
+        <is>
+          <t>Flujo de caja y ciclos de ingreso</t>
+        </is>
+      </c>
+      <c r="B61" s="23" t="inlineStr">
+        <is>
+          <t>5.16</t>
+        </is>
+      </c>
+      <c r="C61" s="18" t="inlineStr">
+        <is>
+          <t>Pedir el dinero disponible hoy con contexto y propósito</t>
+        </is>
+      </c>
+      <c r="D61" s="19" t="inlineStr">
+        <is>
+          <t>La pantalla pregunta '¿Cuánto tienes hoy en tu cuenta?' sin explicar por qué Amy necesita esa cifra ni qué dinero debe incluir. Además, saldo en cuenta y dinero realmente disponible pueden ser diferentes si parte del saldo ya está separado para otros propósitos.</t>
+        </is>
+      </c>
+      <c r="E61" s="19" t="inlineStr">
+        <is>
+          <t>Amy debe pedir un punto de partida para organizar el periodo actual, pero la pregunta debe explicar para qué se utilizará y qué monto debe ingresar la usuaria. El dato debe representar el dinero con el que realmente puede contar para el plan actual, evitando duplicar dinero que ya está separado o comprometido.</t>
+        </is>
+      </c>
+      <c r="F61" s="19" t="inlineStr">
+        <is>
+          <t>Como una mujer que está organizando mi dinero hasta el próximo ingreso, quiero entender exactamente qué cifra debo darle a Amy y por qué la necesita, para que el cálculo parta de una cantidad correcta.</t>
+        </is>
+      </c>
+      <c r="G61" s="19" t="inlineStr">
+        <is>
+          <t>Reemplazar la pregunta aislada por una captura contextual. Explicar que Amy necesita saber con cuánto dinero puede contar la usuaria hoy para organizar lo que queda hasta el próximo ingreso. Definir de forma consistente si el dato solicitado es saldo total o dinero disponible y evitar mezclar ambos conceptos. Si se solicita dinero disponible, aclarar que no debe incluir montos que ya estén separados y no puedan utilizarse. Mostrar cómo este dato alimenta el cálculo del plan. Permitir actualizarlo cuando cambie de forma relevante.</t>
+        </is>
+      </c>
+      <c r="H61" s="19" t="inlineStr">
+        <is>
+          <t>No hacer sentir a la usuaria que debe sumar todas sus cuentas si eso no es necesario para la lógica. La instrucción debe ser específica y acompañarse de un ejemplo breve si existe riesgo de interpretación. Evitar pedir información que Amy ya pueda calcular a partir de datos existentes.</t>
+        </is>
+      </c>
+      <c r="I61" s="19" t="inlineStr">
+        <is>
+          <t>Mejorar la calidad del dato inicial y hacer transparente por qué Amy solicita información financiera.</t>
+        </is>
+      </c>
+      <c r="J61" s="19" t="inlineStr">
+        <is>
+          <t>La usuaria sabe qué monto ingresar y entiende cómo Amy lo utilizará para calcular su plan.</t>
+        </is>
+      </c>
+      <c r="K61" s="19" t="inlineStr">
+        <is>
+          <t>La pregunta define claramente qué dinero incluir, explica su propósito y el valor alimenta correctamente el cálculo hasta el próximo ingreso.</t>
+        </is>
+      </c>
+      <c r="L61" s="19" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M61" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="84.45" customFormat="1" customHeight="1" s="17">
+      <c r="A62" s="18" t="inlineStr">
+        <is>
+          <t>Flujo de caja y ciclos de ingreso</t>
+        </is>
+      </c>
+      <c r="B62" s="23" t="inlineStr">
+        <is>
+          <t>5.17</t>
+        </is>
+      </c>
+      <c r="C62" s="18" t="inlineStr">
+        <is>
+          <t>Hacer autoexplicativos los campos según la frecuencia de ingreso</t>
+        </is>
+      </c>
+      <c r="D62" s="19" t="inlineStr">
+        <is>
+          <t>Al seleccionar una frecuencia como quincenal, la interfaz muestra campos numéricos adicionales sin explicar claramente qué representa cada uno. Por ejemplo, pueden aparecer dos cajas con 15 y 30 sin etiquetas suficientes, obligando a la usuaria a deducir que corresponden a días de pago.</t>
+        </is>
+      </c>
+      <c r="E62" s="19" t="inlineStr">
+        <is>
+          <t>Cada campo que aparezca como consecuencia de la frecuencia seleccionada debe indicar de forma explícita qué información espera Amy. Para ingresos quincenales, la usuaria debe identificar claramente el primer pago y el segundo pago, junto con el día y monto de cada uno.</t>
+        </is>
+      </c>
+      <c r="F62" s="19" t="inlineStr">
+        <is>
+          <t>Como una mujer que está configurando un ingreso quincenal, quiero que cada campo me diga exactamente qué debo ingresar, para completar la información sin tener que adivinar qué significan los números.</t>
+        </is>
+      </c>
+      <c r="G62" s="19" t="inlineStr">
+        <is>
+          <t>Generar campos dinámicos con etiquetas y estructura según la frecuencia elegida. Para quincenal, presentar dos grupos diferenciados: 'Primer pago' con 'Día en que lo recibes' y 'Cuánto recibes', y 'Segundo pago' con los mismos campos. Para otras frecuencias, adaptar el número y tipo de campos necesarios. Nunca mostrar inputs numéricos sin etiqueta o contexto. Integrar esta estructura con la lógica definida en 5.2 para que cada fecha tenga su monto propio.</t>
+        </is>
+      </c>
+      <c r="H62" s="19" t="inlineStr">
+        <is>
+          <t>Las etiquetas deben permanecer visibles aunque el campo tenga contenido. No depender únicamente de placeholders. Mantener una estructura repetible para que la usuaria entienda el segundo bloque después de completar el primero. Aplicar formato monetario global a los campos de monto.</t>
+        </is>
+      </c>
+      <c r="I62" s="19" t="inlineStr">
+        <is>
+          <t>Reducir errores de configuración y hacer que el onboarding de ingresos sea comprensible sin asistencia.</t>
+        </is>
+      </c>
+      <c r="J62" s="19" t="inlineStr">
+        <is>
+          <t>La usuaria completa correctamente fechas y montos porque entiende qué representa cada campo.</t>
+        </is>
+      </c>
+      <c r="K62" s="19" t="inlineStr">
+        <is>
+          <t>Todos los campos dinámicos tienen etiquetas explícitas, la estructura cambia de forma coherente según la frecuencia y no existen inputs cuyo significado deba inferirse.</t>
+        </is>
+      </c>
+      <c r="L62" s="19" t="inlineStr">
+        <is>
+          <t>Alta</t>
+        </is>
+      </c>
+      <c r="M62" s="19" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:O1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: marcar 5.1 y 5.2 como Completo
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/roadmap/Finance-BFF-Experience-Roadmap.xlsx
+++ b/docs/roadmap/Finance-BFF-Experience-Roadmap.xlsx
@@ -3608,7 +3608,7 @@
       </c>
       <c r="M46" s="16" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completo</t>
         </is>
       </c>
     </row>
@@ -3675,7 +3675,7 @@
       </c>
       <c r="M47" s="19" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Completo</t>
         </is>
       </c>
     </row>

</xml_diff>